<commit_message>
Sync FY2026 focus checklists with Hanul DB 2026-07-16 updates.
Load enriched audit-standard and QC reference columns from xlsx, add 15 supplemental checklist rows, and refresh cloud template workbooks.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/templates/4대중점_체크리스트_상장_FY2026.xlsx
+++ b/data/templates/4대중점_체크리스트_상장_FY2026.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="범례" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'체크리스트'!$A$1:$Y$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'체크리스트'!$A$1:$AD$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +45,13 @@
       <name val="맑은 고딕"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -80,7 +85,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF4E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3E9FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -115,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -125,16 +140,22 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -144,6 +165,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -511,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -522,91 +549,98 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>4대 중점 감리 체크리스트 — 금융감독원(상장)</t>
+          <t>4대 중점 감리 체크리스트(고도화) — 금융감독원(상장)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>출처: Hanul DB / 4대 중점사항 감리대상 / 2026년 보도자료 회계위반·오류 예시</t>
+          <t>출처: Hanul DB / 4대 중점사항 감리대상 / 2026년 보도자료 회계위반·오류 예시 + 감리지적사례·회계기준·질의회신·QC 심리점검표 보강</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>용도: 감사조서 자가검토(hanul-002) · 인간 회계사 검토·보완용 living document</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+          <t>용도: 감사조서 자가검토(hanul-002) · 인간 회계사 검토·보완용 living document (고도화판)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>고도화 방법: 기존 checklist_id·golden_set_ids·detect_all/any·red_flag_phrases 등 탐지 로직은 그대로 보존(라이브 룰엔진·골든셋 회귀 호환)하고, review_procedure·basis·to_be 등 서술필드를 심화하며 5개 컬럼(문단 인용·감사기준·추가사례·질의회신·QC연계)을 신설 추가</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>이슈</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>제목</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>체크 항목 수</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>국외 매출·매출채권 회계처리</t>
         </is>
       </c>
-      <c r="C6" t="n">
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>재고자산 평가손실 인식의 적정성</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>투자부동산 회계처리</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
         <v>4</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>재고자산 평가손실 인식의 적정성</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>투자부동산 회계처리</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>충당부채의 인식·측정과 우발부채 공시</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>3</v>
+      <c r="C10" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -620,34 +654,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y18"/>
+  <dimension ref="A1:AD26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="42" customWidth="1" min="22" max="22"/>
-    <col width="36" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="24" customWidth="1" min="25" max="25"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="40" customWidth="1" min="22" max="22"/>
+    <col width="32" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="34" customWidth="1" min="26" max="26"/>
+    <col width="26" customWidth="1" min="27" max="27"/>
+    <col width="34" customWidth="1" min="28" max="28"/>
+    <col width="26" customWidth="1" min="29" max="29"/>
+    <col width="30" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -776,1906 +815,3360 @@
           <t>na_condition</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="7" t="n">
+      <c r="Z1" s="7" t="inlineStr">
+        <is>
+          <t>standard_paragraphs</t>
+        </is>
+      </c>
+      <c r="AA1" s="7" t="inlineStr">
+        <is>
+          <t>audit_standard_ref</t>
+        </is>
+      </c>
+      <c r="AB1" s="7" t="inlineStr">
+        <is>
+          <t>additional_case_refs</t>
+        </is>
+      </c>
+      <c r="AC1" s="7" t="inlineStr">
+        <is>
+          <t>qna_refs</t>
+        </is>
+      </c>
+      <c r="AD1" s="7" t="inlineStr">
+        <is>
+          <t>qc_checklist_ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>국외 매출·매출채권 회계처리</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>L1-01</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>인도조건별 수익인식 시점 검토</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t>매출 과대계상</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 A사</t>
-        </is>
-      </c>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>FOB 선적시점 인식 — 실제 인도·대리점 공급 시점과 불일치</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 A사</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>해외 대리점을 통해 해외 병원에 의료기기를 공급하면서, 대리점 계약에 따라 대리점이 실제 병원에 제품을 공급한 시점에 매출을 인식하여야 함에도 인도조건(FOB)에 따라 제품 선적시점에 매출을 인식하여 매출 과대계상</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>수출·국외매출 유의 시</t>
         </is>
       </c>
-      <c r="J2" s="8" t="inlineStr">
+      <c r="J2" s="9" t="inlineStr">
         <is>
           <t>인도</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t>FOB; 선적; 수행의무; 통제; 수익인식; 인도조건</t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>인도조건; 수익인식 시점</t>
         </is>
       </c>
-      <c r="M2" s="8" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t>인도조건; 통제 이전; 수행의무</t>
         </is>
       </c>
-      <c r="N2" s="8" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t>선적만; FOB만</t>
         </is>
       </c>
-      <c r="O2" s="8" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1115호</t>
         </is>
       </c>
-      <c r="P2" s="8" t="inlineStr">
-        <is>
-          <t>인도조건·수행의무 이행 시점 및 검토 결론 문서화</t>
-        </is>
-      </c>
-      <c r="Q2" s="8" t="inlineStr">
-        <is>
-          <t>인도조건 판단 근거·결론 보강(통제 이전 시점 명시)</t>
-        </is>
-      </c>
-      <c r="R2" s="8" t="inlineStr"/>
-      <c r="S2" s="8" t="inlineStr">
+      <c r="P2" s="9" t="inlineStr">
+        <is>
+          <t>인도조건(FOB/DDP/DAP/CIF 등)별 수행의무 이행시점 및 검토 결론을 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q2" s="9" t="inlineStr">
+        <is>
+          <t>인도조건 판단 근거·결론(통제 이전 시점 명시)을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R2" s="9" t="inlineStr"/>
+      <c r="S2" s="9" t="inlineStr">
         <is>
           <t>매출채권; 매출</t>
         </is>
       </c>
-      <c r="T2" s="8" t="inlineStr">
+      <c r="T2" s="9" t="inlineStr">
         <is>
           <t>국외; 해외; 수출; 외화; 매출채권; 외상매출</t>
         </is>
       </c>
-      <c r="U2" s="8" t="inlineStr">
+      <c r="U2" s="9" t="inlineStr">
         <is>
           <t>C; P</t>
         </is>
       </c>
-      <c r="V2" s="8" t="inlineStr">
-        <is>
-          <t>① C·P Lead에서 국외·수출 거래 목록·인도조건(FOB/CIF 등) 확인 ② 수행의무 이행·통제 이전 시점과 매출 인식 시점 대사 ③ 선적일만 근거로 인식한 거래·대리점 경유 거래 식별 ④ 인도조건 판단 근거·결론 문장 기재 여부 확인</t>
-        </is>
-      </c>
-      <c r="W2" s="8" t="inlineStr">
-        <is>
-          <t>FOB 선적 시점만으로 수익을 인식했는가?; 실제 인도·통제 이전 시점과 인식 시점이 일치하는가?; 인도조건별 수행의무 이행 근거가 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X2" s="8" t="inlineStr"/>
-      <c r="Y2" s="8" t="inlineStr"/>
-    </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="7" t="n">
+      <c r="V2" s="9" t="inlineStr">
+        <is>
+          <t>① C·P Lead에서 국외·수출 거래 목록·인도조건(FOB/CIF/DDP/DAP 등) 확인 ② 수행의무 이행·통제 이전 시점과 매출 인식 시점 대사 ③ 선적일만 근거로 인식한 거래·대리점 경유 거래 식별 ④ DDP·DAP 등 도착지인도조건에서 '도착일 추적이 어렵다'는 사유로 선적일 기준 인식하지 않았는지 점검 ⑤ 인도조건 판단 근거·결론 문장 기재 여부 확인</t>
+        </is>
+      </c>
+      <c r="W2" s="9" t="inlineStr">
+        <is>
+          <t>FOB 선적 시점만으로 수익을 인식했는가?; 실제 인도·통제 이전 시점과 인식 시점이 일치하는가?; 인도조건별 수행의무 이행 근거가 문서화되어 있는가?; DDP·DAP 등 도착지인도조건 거래를 도착일 확인 곤란을 이유로 선적일에 인식하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X2" s="9" t="inlineStr"/>
+      <c r="Y2" s="9" t="inlineStr"/>
+      <c r="Z2" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 16.10·결16.7(경제적 실질 우선), K-IFRS 1115호 문단29·31·33(결합수행의무 판단), 문단38(통제이전 지표)</t>
+        </is>
+      </c>
+      <c r="AA2" s="11" t="inlineStr">
+        <is>
+          <t>KSA 240 문단32-33(경영진 통제 무력화, 수익인식 부정위험 추정), KSA 330(위험대응)</t>
+        </is>
+      </c>
+      <c r="AB2" s="11" t="inlineStr">
+        <is>
+          <t>KICPA-2025-06(자동차 엔진부품 제조사, DDP·DAP 조건임에도 도착일 추적 어렵다는 사유로 선적일 인식); FSS2405-06(납품·설치계약을 형식상 분리해 결합수행의무 오판, 조기 매출인식)</t>
+        </is>
+      </c>
+      <c r="AC2" s="11" t="inlineStr">
+        <is>
+          <t>신속처리질의 선적지인도조건(FOB) 수입 회계처리(참고); GKQA01-037(수출대행계약에 따른 매출시 계정분류 — 순액인식)</t>
+        </is>
+      </c>
+      <c r="AD2" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목31·32 수익인식('25비상장테마 국외매출 회계처리, P): 주요 매출유형별 수익인식기준 적정성 미검토, 발생사실TEST증빙이 세금계산서에 한정된 경우 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>국외 매출·매출채권 회계처리</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>L1-02</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>허위·가공 매출 여부 검토</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>허위 매출</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 B사</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>허위 계약·수출신고필증 위변조 등 실질 납품 없는 매출</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 B사</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>해외 종속회사를 통해 해외에 제품을 납품한다는 허위 사실을 공시하고, 허위의 매출·매입 계약서 작성, 수출입신고필증 위·변조 등의 방법으로 제품을 실제 납품한 것처럼 가장하여 매출 및 매출원가를 허위계상</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr"/>
-      <c r="J3" s="8" t="inlineStr"/>
-      <c r="K3" s="8" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr"/>
+      <c r="J3" s="9" t="inlineStr"/>
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t>허위; 위변조; 수출입; 실질; 납품</t>
         </is>
       </c>
-      <c r="L3" s="8" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>계약; 신고; 증빙</t>
         </is>
       </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>실질; 증빙; 납품 확인</t>
         </is>
       </c>
-      <c r="N3" s="8" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t>허위; 가공</t>
         </is>
       </c>
-      <c r="O3" s="8" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1115호</t>
         </is>
       </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>국외 매출 실질·증빙 대사 절차 및 결론 기재</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>거래 실질·증빙 검토 내용 보강</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr"/>
-      <c r="S3" s="8" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
+        <is>
+          <t>국외 매출 실질·증빙 대사 절차 및 결론을 문서화 바랍니다(선적서류·물류 입출고 기록·거래상대방 관계 대사 포함)</t>
+        </is>
+      </c>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>거래 실질·증빙 검토 내용을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R3" s="9" t="inlineStr"/>
+      <c r="S3" s="9" t="inlineStr">
         <is>
           <t>매출채권; 매출</t>
         </is>
       </c>
-      <c r="T3" s="8" t="inlineStr">
+      <c r="T3" s="9" t="inlineStr">
         <is>
           <t>국외; 해외; 수출; 외화; 매출채권; 외상매출</t>
         </is>
       </c>
-      <c r="U3" s="8" t="inlineStr">
+      <c r="U3" s="9" t="inlineStr">
         <is>
           <t>C; P</t>
         </is>
       </c>
-      <c r="V3" s="8" t="inlineStr">
-        <is>
-          <t>① 국외 매출 계약·수출신고·납품 증빙 대사 ② 실질 납품 없이 인식된 매출(허위·가공) 여부 점검 ③ 수출입 실적·통관 자료와 장부 대사 ④ 이상 거래에 대한 추가 절차·결론 기재 확인</t>
-        </is>
-      </c>
-      <c r="W3" s="8" t="inlineStr">
-        <is>
-          <t>계약·신고·납품 증빙 없이 인식된 매출이 있는가?; 허위·가공 매출에 대한 실질 검토가 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X3" s="8" t="inlineStr"/>
-      <c r="Y3" s="8" t="inlineStr"/>
-    </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="7" t="n">
+      <c r="V3" s="9" t="inlineStr">
+        <is>
+          <t>① 국외 매출 계약·수출신고·납품 증빙 대사 ② 실질 납품 없이 인식된 매출(허위·가공) 여부 점검 — 무자료업체·자금 순환거래·단순분리 후 재수출 패턴 점검 ③ 수출입 실적·통관 자료와 장부 대사, 신규 해외거래처와의 비정상적 대량거래 여부 확인 ④ 해외거래처 조회서 발송거부·미회신에 대한 대체적 절차(재무제표일 후 대금회수내역 확인 등) 수행 여부 확인 ⑤ 이상 거래에 대한 추가 절차·결론 기재 확인</t>
+        </is>
+      </c>
+      <c r="W3" s="9" t="inlineStr">
+        <is>
+          <t>계약·신고·납품 증빙 없이 인식된 매출이 있는가?; 허위·가공 매출에 대한 실질 검토가 문서화되어 있는가?; 신규 해외거래처와의 비정상적 대량거래에 대해 선적서류·물류기록을 대사하였는가?; 조회서 발송거부·미회신에 대체적 절차를 수행하였는가?</t>
+        </is>
+      </c>
+      <c r="X3" s="9" t="inlineStr"/>
+      <c r="Y3" s="9" t="inlineStr"/>
+      <c r="Z3" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1115호(수익인식 요건 — 계약의 상업적 실질)</t>
+        </is>
+      </c>
+      <c r="AA3" s="11" t="inlineStr">
+        <is>
+          <t>KSA 240 문단30-33(부정으로 인한 수익인식 위험 추정), KSA 505(외부조회 — 수신인 주소 타당성, 대체적 절차)</t>
+        </is>
+      </c>
+      <c r="AB3" s="11" t="inlineStr">
+        <is>
+          <t>FSS2405-04(무자료업체 실물흐름 근거로 계약서·세금계산서·수출신고필증 외관만 구비, 특수관계 미파악); FSS2409-01(홍콩 거래처와 공모해 단순분리 후 재수출로 위장, 자금 순환구조); KICPA-2025-45/46(총괄표·부가세신고서 대사만으로 발생사실·기간귀속 확인 대체)</t>
+        </is>
+      </c>
+      <c r="AC3" s="11" t="inlineStr"/>
+      <c r="AD3" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목31·32: MUS 미사용, 발생사실TEST증빙이 세금계산서에 한정, 기간귀속테스트 샘플선정근거 미기재 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>국외 매출·매출채권 회계처리</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>L1-03</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>국외 매출채권 ECL(손실충당금) 측정</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>ECL 미계상</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 C사</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>종속 해외채권에 손실충당금 미설정</t>
-        </is>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 C사</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>지배기업이 종속기업의 해외거래처 매출채권이 지배기업과 유사한 거래에서 발생한 매출채권이었음에도, 지배기업의 회계정책(간편법)을 적용하지 않고 종속기업의 해외거래처 매출채권에 대해서는 손실충당금을 설정하지 않아 당기순이익·자기자본 과대계상</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
         <is>
           <t>채권 잔액 중요성 이상</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>신용</t>
         </is>
       </c>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>기대신용손실; 손실충당금; ECL; 12개월; 전체기간</t>
         </is>
       </c>
-      <c r="L4" s="8" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>ECL; 신용위험</t>
         </is>
       </c>
-      <c r="M4" s="8" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>기대신용손실; 손실충당금; 간편법</t>
         </is>
       </c>
-      <c r="N4" s="8" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>충당 미설정; ECL 없음</t>
         </is>
       </c>
-      <c r="O4" s="8" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1109호</t>
         </is>
       </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>신용위험 증가 평가·ECL 산정 및 결론 문서화</t>
-        </is>
-      </c>
-      <c r="Q4" s="8" t="inlineStr">
-        <is>
-          <t>ECL 모형·가정 및 손실충당금 결론 보강</t>
-        </is>
-      </c>
-      <c r="R4" s="8" t="inlineStr"/>
-      <c r="S4" s="8" t="inlineStr">
+      <c r="P4" s="9" t="inlineStr">
+        <is>
+          <t>신용위험 유의적 증가 평가·ECL 산정 및 결론을 문서화 바랍니다(완전자본잠식 등 손상징후가 있는 종속회사 채권을 '종속회사'라는 이유로 검토 생략하지 않았는지 포함)</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>ECL 모형·가정 및 손실충당금 결론(연체전이율 등)을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R4" s="9" t="inlineStr"/>
+      <c r="S4" s="9" t="inlineStr">
         <is>
           <t>매출채권; 매출</t>
         </is>
       </c>
-      <c r="T4" s="8" t="inlineStr">
+      <c r="T4" s="9" t="inlineStr">
         <is>
           <t>국외; 해외; 수출; 외화; 매출채권; 외상매출</t>
         </is>
       </c>
-      <c r="U4" s="8" t="inlineStr">
+      <c r="U4" s="9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="V4" s="8" t="inlineStr">
-        <is>
-          <t>① C Lead에서 국외·종속 해외채권 잔액·연령 확인 ② 신용위험 유의적 증가 평가(12개월/전체기간 ECL) 문서화 ③ 손실충당금 산정 모형·가정·결론 확인 ④ '기대신용손실 반영 완료' 등 인정문장 기재</t>
-        </is>
-      </c>
-      <c r="W4" s="8" t="inlineStr">
-        <is>
-          <t>국외·종속 해외채권에 ECL이 계상되어 있는가?; 신용위험 증가 평가 및 손실충당금 산정 근거가 있는가?</t>
-        </is>
-      </c>
-      <c r="X4" s="8" t="inlineStr"/>
-      <c r="Y4" s="8" t="inlineStr"/>
-    </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="7" t="n">
+      <c r="V4" s="9" t="inlineStr">
+        <is>
+          <t>① C Lead에서 국외·종속 해외채권 잔액·연령 확인 ② 신용위험 유의적 증가 평가(12개월/전체기간 ECL) 문서화, 지배기업 회계정책(간편법)이 종속기업 채권에도 일관 적용되는지 확인 ③ 완전자본잠식·생산중단 등 손상징후가 있는 종속회사 매출채권을 '신사업계획상 매출 예정' 등 사유로 미설정하지 않았는지 점검 ④ 연체기간별 충당률·연체전이율(Roll-rate) 적용 및 외화환산손익과의 혼동 여부 확인 ⑤ 손실충당금 산정 모형·가정·결론 확인, '기대신용손실 반영 완료' 등 인정문장 기재</t>
+        </is>
+      </c>
+      <c r="W4" s="9" t="inlineStr">
+        <is>
+          <t>국외·종속 해외채권에 ECL이 계상되어 있는가?; 신용위험 증가 평가 및 손실충당금 산정 근거가 있는가?; 완전자본잠식 종속회사 매출채권을 별도재무제표에서 독립적으로 손상평가하였는가?; 환율변동 손실충당금 변동분을 손상차손이 아닌 외환차이로 구분하였는가?</t>
+        </is>
+      </c>
+      <c r="X4" s="9" t="inlineStr"/>
+      <c r="Y4" s="9" t="inlineStr"/>
+      <c r="Z4" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1109호 문단5.5.4·5.5.8·5.5.17(기대신용손실·미래전망정보), 1039호 문단58·59(손상의 객관적 증거, 구기준 참고); 일반기업회계기준 6.17의2(K-GAAP 발생손실모형은 ECL과 달리 손상의 객관적 증거·회수불확실성 요구)</t>
+        </is>
+      </c>
+      <c r="AA4" s="11" t="inlineStr">
+        <is>
+          <t>KSA 540(회계추정치 감사 — ECL 모형·가정·데이터 평가), KSA 560(후속사건 — 발행승인일 전 매출처 파산은 수정요 사건)</t>
+        </is>
+      </c>
+      <c r="AB4" s="11" t="inlineStr">
+        <is>
+          <t>FSS1912-10(피혁 자회사 5년 연속 순손실·완전자본잠식임에도 종속회사라는 이유로 손상검토 생략, 별도FS 손상평가 판단기준 제시); KICPA-2022-07(중국 종속기업 생산중단·완전자본잠식에도 신사업계획 이유로 미설정); FSS2505-09(1년 초과 연체를 일부회수중이라는 사유로 미연체 분류); FSS2311-15(외화환산손익과 손실충당금 혼동으로 연체전이율 오염)</t>
+        </is>
+      </c>
+      <c r="AC4" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 외화 매출채권에 대한 대손충당금 환산(환율변동 대손충당금 변동분은 손상차손이 아닌 외환차이, K-IFRS1109 IE98~99); 손실충당금과 보고기간후사건(발행승인일전 매출처 파산은 수정요 사건, 1010호 문단9⑵㈎)</t>
+        </is>
+      </c>
+      <c r="AD4" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목26 수취채권(C,'25비상장테마 매출채권 대손충당금): 대손충당금 검토내역 부실기재 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>국외 매출·매출채권 회계처리</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>L1-04</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>환율·지정학 리스크 반영</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t>거시요인 미반영</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>금감원 유의사항 ③</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>환율·수출입 제한 등이 ECL에 미반영</t>
-        </is>
-      </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>지정학적 리스크, 수출입 제한, 환율 변동 등 거시적 요인이 채무불이행 위험에 미치는 영향을 평가하여 손실충당금 산정에 반영하지 않음</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr"/>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr"/>
+      <c r="J5" s="9" t="inlineStr">
         <is>
           <t>환율</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>지정학; 수출입; 외화; 변동성</t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>환율; 리스크</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>지정학; 거시; 채무불이행</t>
         </is>
       </c>
-      <c r="N5" s="8" t="inlineStr"/>
-      <c r="O5" s="8" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr"/>
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1109호; 1021호</t>
         </is>
       </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>거시요인이 ECL에 반영되었는지 검토 기재</t>
-        </is>
-      </c>
-      <c r="Q5" s="8" t="inlineStr">
-        <is>
-          <t>환율·지정학 요인 평가 결론 보강</t>
-        </is>
-      </c>
-      <c r="R5" s="8" t="inlineStr"/>
-      <c r="S5" s="8" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
+        <is>
+          <t>거시요인이 ECL에 반영되었는지 검토를 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>환율·지정학 요인 평가 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R5" s="9" t="inlineStr"/>
+      <c r="S5" s="9" t="inlineStr">
         <is>
           <t>매출채권; 매출</t>
         </is>
       </c>
-      <c r="T5" s="8" t="inlineStr">
+      <c r="T5" s="9" t="inlineStr">
         <is>
           <t>국외; 해외; 수출; 외화; 매출채권; 외상매출</t>
         </is>
       </c>
-      <c r="U5" s="8" t="inlineStr">
+      <c r="U5" s="9" t="inlineStr">
         <is>
           <t>C; P</t>
         </is>
       </c>
-      <c r="V5" s="8" t="inlineStr">
-        <is>
-          <t>① 환율·지정학·수출입 제한 등 거시요인이 ECL에 반영되었는지 확인 ② 외화환산·cut-off와 연계 검토 ③ 거시요인 평가 결론·민감도 분석 문서화</t>
-        </is>
-      </c>
-      <c r="W5" s="8" t="inlineStr">
-        <is>
-          <t>환율·지정학 리스크가 ECL 산정에 반영되었는가?; 거시요인 평가 결론이 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X5" s="8" t="inlineStr"/>
-      <c r="Y5" s="8" t="inlineStr"/>
-    </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="11" t="n">
+      <c r="V5" s="9" t="inlineStr">
+        <is>
+          <t>① 환율·지정학·수출입 제한 등 거시요인이 ECL에 반영되었는지 확인 ② 환위험 헷지 목적이라는 회사 주장(제3자 경유 원화 회수 등)을 검증 없이 수용하지 않았는지 점검 ③ 외화환산·cut-off와 연계 검토 ④ 거시요인 평가 결론·민감도 분석 문서화</t>
+        </is>
+      </c>
+      <c r="W5" s="9" t="inlineStr">
+        <is>
+          <t>환율·지정학 리스크가 ECL 산정에 반영되었는가?; 거시요인 평가 결론이 문서화되어 있는가?; 환위험 헷지 주장을 검증 없이 그대로 수용하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X5" s="9" t="inlineStr"/>
+      <c r="Y5" s="9" t="inlineStr"/>
+      <c r="Z5" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 제23장(환율변동효과)</t>
+        </is>
+      </c>
+      <c r="AA5" s="11" t="inlineStr">
+        <is>
+          <t>KSA 540(회계추정 감사 — 거시경제 가정의 합리성 평가)</t>
+        </is>
+      </c>
+      <c r="AB5" s="11" t="inlineStr">
+        <is>
+          <t>FSS2405-04(환위험 헷지 목적으로 제3자를 통해 원화 회수한다는 회사 주장을 검증 없이 수용); KICPA-2025-06(관세·통관 리스크가 인도시점 판단에 영향)</t>
+        </is>
+      </c>
+      <c r="AC5" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 외화 매출채권에 대한 대손충당금 환산(공유)</t>
+        </is>
+      </c>
+      <c r="AD5" s="11" t="inlineStr"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>국외 매출·매출채권 회계처리</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>L1-05</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>본인·대리인(총액/순액) 판단 및 특수관계자 매출채권 우회회수·상계</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>총액·순액 인식 오류, 채권 우회회수</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>금감원·한공회 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>해외 특수관계자 거래에서 주된책임·재고위험·가격결정권 등 통제지표를 충족하지 못함에도 총액으로 수익을 인식(대리인임에도 본인으로 오판), 또는 우회 회수된 해외매출채권을 관계사차입금·채무면제이익으로 위장하여 장부에서 제거하지 않음</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>결론미비</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>해외 특수관계자 거래 유의 시</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr"/>
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>본인; 대리인; 총액; 순액; 통제지표; 우회회수</t>
+        </is>
+      </c>
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>통제지표 검토</t>
+        </is>
+      </c>
+      <c r="M6" s="9" t="inlineStr">
+        <is>
+          <t>주된책임; 재고위험; 가격결정권 검토</t>
+        </is>
+      </c>
+      <c r="N6" s="9" t="inlineStr">
+        <is>
+          <t>우회 회수; 채무면제이익 위장</t>
+        </is>
+      </c>
+      <c r="O6" s="9" t="inlineStr">
+        <is>
+          <t>K-IFRS 1115호</t>
+        </is>
+      </c>
+      <c r="P6" s="9" t="inlineStr">
+        <is>
+          <t>해외 특수관계자 거래에 대해 통제지표(주된책임/재고위험/가격결정권) 3요소를 검토하여 총액·순액 인식의 타당성을 확인하고, 매출채권 우회회수·상계 여부를 검토 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
+        <is>
+          <t>통제지표 판단 근거 및 채권 제거·상계 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R6" s="9" t="inlineStr"/>
+      <c r="S6" s="9" t="inlineStr">
+        <is>
+          <t>매출채권; 매출</t>
+        </is>
+      </c>
+      <c r="T6" s="9" t="inlineStr">
+        <is>
+          <t>국외; 해외; 수출; 외화; 매출채권; 외상매출</t>
+        </is>
+      </c>
+      <c r="U6" s="9" t="inlineStr">
+        <is>
+          <t>C; P</t>
+        </is>
+      </c>
+      <c r="V6" s="9" t="inlineStr">
+        <is>
+          <t>① 해외 관계사(3자거래 포함) 거래에 대해 통제지표(주된책임·재고위험·가격결정권, K-IFRS1115 문단B34~B38) 검토 ② 수출업무 대행자에 불과함에도 총액인식하지 않았는지 확인 ③ 우회 회수된 해외매출채권이 관계사차입금 전환·채무면제이익 등으로 위장되어 장부에서 제거되지 않았는지 확인 ④ 결론 문서화</t>
+        </is>
+      </c>
+      <c r="W6" s="9" t="inlineStr">
+        <is>
+          <t>해외 관계사 거래에 대해 통제지표(주된책임/재고위험/가격결정권) 3요소를 검토하였는가?; 우회 회수된 매출채권이 관계사차입금·채무면제이익 등으로 위장되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X6" s="9" t="inlineStr"/>
+      <c r="Y6" s="9" t="inlineStr">
+        <is>
+          <t>본인·대리인 판단이 필요한 3자 거래 또는 해외 특수관계자 거래가 없는 경우</t>
+        </is>
+      </c>
+      <c r="Z6" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1115호 문단33·B34~B38(통제지표), 일반기업회계기준 16.8·16.10·실16.19</t>
+        </is>
+      </c>
+      <c r="AA6" s="11" t="inlineStr">
+        <is>
+          <t>KSA 550(특수관계자), KSA 240 문단32-33</t>
+        </is>
+      </c>
+      <c r="AB6" s="11" t="inlineStr">
+        <is>
+          <t>FSS2505-03(미국 손자회사 3자거래, 3대 통제지표 모두 미충족에도 총액인식); FSS2409-02(협력업체 상품매출 본인/대리인 오판); KICPA-2025-30(해외 특수관계자가 가격·사양·배송 책임 모두 부담함에도 총액인식); KICPA-2025-28(우회 회수된 해외매출채권을 관계사차입금·채무면제이익으로 위장)</t>
+        </is>
+      </c>
+      <c r="AC6" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 종속기업이 대리인일 때 특수관계자와의 거래 금액(순액 공시); 유상사급 거래의 수익 인식(총액 vs 순액, 1115호 문단33·38); 수출대행계약에 따른 매출시 계정분류(순액 인식)</t>
+        </is>
+      </c>
+      <c r="AD6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>국외 매출·매출채권 회계처리</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>L1-06</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>매출·매출채권 감사증거 편중 및 대체적 절차 수행</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>감사절차 편중·대체절차 미실시</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>한공회 QC 심리점검표·금감원 감리지적사례</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>발생사실·기간귀속 테스트를 총괄표·부가세신고서 대사로만 대체하거나 세금계산서에 한정된 증빙만으로 발생사실을 확인, 해외거래처 조회서 미회신·발송거부에 대체적 절차를 수행하지 않음</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>검토누락</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr"/>
+      <c r="J7" s="9" t="inlineStr"/>
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>발생사실TEST; 기간귀속; MUS; 대체적 절차; 외부조회</t>
+        </is>
+      </c>
+      <c r="L7" s="9" t="inlineStr">
+        <is>
+          <t>발생사실 테스트 증빙</t>
+        </is>
+      </c>
+      <c r="M7" s="9" t="inlineStr">
+        <is>
+          <t>MUS 사용; 대체적 절차 수행; 선적서류 대사</t>
+        </is>
+      </c>
+      <c r="N7" s="9" t="inlineStr">
+        <is>
+          <t>세금계산서에 한정; 대체절차 없음</t>
+        </is>
+      </c>
+      <c r="O7" s="9" t="inlineStr">
+        <is>
+          <t>회계감사기준서 505; 330</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="inlineStr">
+        <is>
+          <t>해외 매출채권 외부조회 미회신 건에 대한 대체적 절차, 발생사실·기간귀속 테스트의 표본추출근거를 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>발생사실 테스트 증빙(선적서류·계약서·입금내역 교차검증)과 대체적 절차 수행 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R7" s="9" t="inlineStr"/>
+      <c r="S7" s="9" t="inlineStr">
+        <is>
+          <t>매출채권; 매출</t>
+        </is>
+      </c>
+      <c r="T7" s="9" t="inlineStr">
+        <is>
+          <t>국외; 해외; 수출; 외화; 매출채권; 외상매출</t>
+        </is>
+      </c>
+      <c r="U7" s="9" t="inlineStr">
+        <is>
+          <t>C; P</t>
+        </is>
+      </c>
+      <c r="V7" s="9" t="inlineStr">
+        <is>
+          <t>① 발생사실·기간귀속 테스트 수행 여부 확인, MUS 등 표본추출방법의 적정성 확인 ② 발생사실 테스트 증빙이 세금계산서에 한정되지 않고 선적서류·계약서·입금내역과 교차검증되었는지 확인 ③ 해외 매출채권 외부조회 미회신 건에 대해 재무제표일 후 대금회수내역 확인 등 대체적 절차 수행 여부 확인 ④ 회사가 조회서를 직접 발송·회수하지 않고 감사인이 통제를 유지하였는지 확인</t>
+        </is>
+      </c>
+      <c r="W7" s="9" t="inlineStr">
+        <is>
+          <t>발생사실 테스트 증빙을 세금계산서에 한정하지 않고 선적서류·계약서·입금내역과 교차검증하였는가?; 외부조회 미회신 건에 대체적 절차를 수행하였는가?; 조회서 발송·회수를 감사인이 통제하였는가?</t>
+        </is>
+      </c>
+      <c r="X7" s="9" t="inlineStr"/>
+      <c r="Y7" s="9" t="inlineStr"/>
+      <c r="Z7" s="11" t="inlineStr"/>
+      <c r="AA7" s="11" t="inlineStr">
+        <is>
+          <t>KSA 505(외부조회 — 수신인 주소 타당성, 대체적 절차), KSA 330(세부테스트 필수), KSA 540, KSA 240(수익인식 부정위험 가정)</t>
+        </is>
+      </c>
+      <c r="AB7" s="11" t="inlineStr">
+        <is>
+          <t>KICPA-2025-45/46(총괄표·부가세신고서 대사만으로 발생사실·기간귀속·회수가능성 확인 대체); FSS2409-10(외부조회 수신인 주소 타당성 미검증, 회사 직원이 조회서 직접 발송·회수); FSS2505-01(해외거래처 조회서 발송거부를 이유로 외부조회 생략); KICPA-2025-09(미회신 매출채권 대체적 절차·대손충당금 검토 소홀)</t>
+        </is>
+      </c>
+      <c r="AC7" s="11" t="inlineStr"/>
+      <c r="AD7" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목31·32(공유): 발생사실TEST에 MUS 미사용, 발생사실 TEST의 증빙이 세금계산서에 한정, 기간귀속 테스트 샘플 선정근거 미기재 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>L2-01</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>항목별 저가법·NRV 평가</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>항목별 평가 오류</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 D사</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>제품군 묶음 평가·일부 재고만 평가손실</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 D사</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>지속적으로 매출총손실이 발생하는 등 원가 회수가능성이 현저히 감소하였음에도 '1년 이상 이동이 없는 재고'에 대해서만 평가손실을 인식하고, 세부 항목 구분이 가능함에도 제품군을 묶어서 평가하여 재고자산 평가손실 과소계상</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I8" s="9" t="inlineStr">
         <is>
           <t>재고 중요성 이상</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J8" s="9" t="inlineStr">
         <is>
           <t>저가법</t>
         </is>
       </c>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="K8" s="9" t="inlineStr">
         <is>
           <t>NRV; 순실현; 항목별; 품목별; 평가손실</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>저가법; NRV</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>항목별; 품목별; 평가손실</t>
         </is>
       </c>
-      <c r="N6" s="8" t="inlineStr">
+      <c r="N8" s="9" t="inlineStr">
         <is>
           <t>제품군만; 이동없는</t>
         </is>
       </c>
-      <c r="O6" s="8" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호</t>
         </is>
       </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>항목별 NRV 산정·평가손실 인식 검토 문서화</t>
-        </is>
-      </c>
-      <c r="Q6" s="8" t="inlineStr">
-        <is>
-          <t>항목별 평가 근거·결론 보강</t>
-        </is>
-      </c>
-      <c r="R6" s="8" t="inlineStr">
+      <c r="P8" s="9" t="inlineStr">
+        <is>
+          <t>항목별 NRV 산정·평가손실 인식 검토를 문서화 바랍니다(차종·사업부 등으로 통합평가하지 않았는지 포함)</t>
+        </is>
+      </c>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>항목별 평가 근거·결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R8" s="9" t="inlineStr">
         <is>
           <t>GS-F-L2-01</t>
         </is>
       </c>
-      <c r="S6" s="8" t="inlineStr">
+      <c r="S8" s="9" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="T6" s="8" t="inlineStr">
+      <c r="T8" s="9" t="inlineStr">
         <is>
           <t>재고; 저가법; 평가손실; 순실현</t>
         </is>
       </c>
-      <c r="U6" s="8" t="inlineStr">
+      <c r="U8" s="9" t="inlineStr">
         <is>
           <t>E; E100</t>
         </is>
       </c>
-      <c r="V6" s="8" t="inlineStr">
-        <is>
-          <t>① E Lead·세부조서에서 품목별 NRV 산정표·저가법 적용 확인 ② 평가손실 인식 품목·금액·근거 문서화 ③ 제품군 일괄평가·일부 품목만 평가 등 red flag 점검 ④ '항목별 NRV 산정·평가손실 인식' 결론문 기재</t>
-        </is>
-      </c>
-      <c r="W6" s="8" t="inlineStr">
-        <is>
-          <t>저가법이 항목별로 적용되었는가?; NRV 산정 및 평가손실 인식 결론이 구체적으로 기재되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X6" s="8" t="inlineStr"/>
-      <c r="Y6" s="8" t="inlineStr"/>
-    </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="11" t="n">
+      <c r="V8" s="9" t="inlineStr">
+        <is>
+          <t>① E Lead·세부조서에서 품목별 NRV 산정표·저가법 적용 확인 ② 차종별·사업부별·제품군별로 일괄 통합평가하여 일부 그룹에서만 평가손실을 인식하지 않았는지 점검(항목별 구분 가능 여부 확인) ③ 평가손실 인식 품목·금액·근거 문서화 ④ 원가율 낮음 등 임의기준으로 특정 품목을 평가대상에서 제외하지 않았는지 확인 ⑤ '항목별 NRV 산정·평가손실 인식' 결론문 기재</t>
+        </is>
+      </c>
+      <c r="W8" s="9" t="inlineStr">
+        <is>
+          <t>저가법이 항목별로 적용되었는가?; NRV 산정 및 평가손실 인식 결론이 구체적으로 기재되어 있는가?; 차종·사업부·제품군 단위로 통합평가하여 일부 그룹만 평가하지 않았는가?; 원가율이 낮다는 이유로 일부 품목을 평가대상에서 제외하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X8" s="9" t="inlineStr"/>
+      <c r="Y8" s="9" t="inlineStr"/>
+      <c r="Z8" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 7.18(저가법은 총액기준 적용 불가), 실무지침 실7.8~실7.9(개별평가 원칙, 통합평가 예외요건); K-IFRS 1002호 문단29</t>
+        </is>
+      </c>
+      <c r="AA8" s="11" t="inlineStr">
+        <is>
+          <t>KSA 501 문단4-8(재고자산 실사입회), KSA 540(NRV 추정치 감사)</t>
+        </is>
+      </c>
+      <c r="AB8" s="11" t="inlineStr">
+        <is>
+          <t>FSS2512-07(차종별로 재고자산을 묶어 부(-)영업손익 발생 차종만 저가법 평가); FSS2311-09(판매가능성 고려 없이 취득 후 5년 경과 단일기준만 적용); KICPA-2020-06(1년이상 2년미만 변동없는 재고 저가법 대상 누락, 원가율 낮은 사업부 재고 NRV평가 제외)</t>
+        </is>
+      </c>
+      <c r="AC8" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 신속처리질의(2022-12-19, 저가법 적용의 회계단위) — 재고자산의 분류나 특정 영업부문에 속하는 모든 재고자산에 기초한 저가법 적용은 부적절</t>
+        </is>
+      </c>
+      <c r="AD8" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목27 재고자산(E): 저가법검토 부적절 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>L2-02</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>진부화·판매부진 재고 평가</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E9" s="9" t="inlineStr">
         <is>
           <t>일부 재고 미평가</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 E사</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>품질문제·단종 재고 평가손실 미인식</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 E사</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>제품 일부 항목이 품질문제로 재고금액의 10%만 판매되는 등 판매가 부진하였고, 일부 항목은 판매가 중단되거나 단종되어 진부화되었음에도 재고자산 평가시 이를 고려하지 않아 재고자산 평가손실 과소계상</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr"/>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="I9" s="9" t="inlineStr"/>
+      <c r="J9" s="9" t="inlineStr">
         <is>
           <t>진부화</t>
         </is>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>판매부진; 단종; 품질; 평가손실</t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
         <is>
           <t>진부화; NRV</t>
         </is>
       </c>
-      <c r="M7" s="8" t="inlineStr">
+      <c r="M9" s="9" t="inlineStr">
         <is>
           <t>평가손실; 순실현</t>
         </is>
       </c>
-      <c r="N7" s="8" t="inlineStr">
+      <c r="N9" s="9" t="inlineStr">
         <is>
           <t>미평가; 취득원가 그대로</t>
         </is>
       </c>
-      <c r="O7" s="8" t="inlineStr">
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호</t>
         </is>
       </c>
-      <c r="P7" s="8" t="inlineStr">
-        <is>
-          <t>진부화·체화 재고 식별 및 평가손실 검토</t>
-        </is>
-      </c>
-      <c r="Q7" s="8" t="inlineStr">
-        <is>
-          <t>판매부진·단종 재고 평가 결론 보강</t>
-        </is>
-      </c>
-      <c r="R7" s="8" t="inlineStr">
+      <c r="P9" s="9" t="inlineStr">
+        <is>
+          <t>진부화·체화 재고 식별 및 평가손실 검토를 문서화 바랍니다(유효기간·품목허가 변경 등 규제상 판매불가 재고, 유통기한 없는 재고 포함)</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>판매부진·단종 재고 평가 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R9" s="9" t="inlineStr">
         <is>
           <t>GS-F-L2-02</t>
         </is>
       </c>
-      <c r="S7" s="8" t="inlineStr">
+      <c r="S9" s="9" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="T7" s="8" t="inlineStr">
+      <c r="T9" s="9" t="inlineStr">
         <is>
           <t>재고; 저가법; 평가손실; 순실현</t>
         </is>
       </c>
-      <c r="U7" s="8" t="inlineStr">
+      <c r="U9" s="9" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="V7" s="8" t="inlineStr">
-        <is>
-          <t>① 진부화·단종·판매부진 재고 식별 절차 확인 ② 해당 재고 NRV·평가손실 인식 여부 ③ 품질문제·체화 재고 목록·금액 대사</t>
-        </is>
-      </c>
-      <c r="W7" s="8" t="inlineStr">
-        <is>
-          <t>진부화·단종 재고가 식별·평가되었는가?; 판매부진 재고에 평가손실이 인식되었는가?</t>
-        </is>
-      </c>
-      <c r="X7" s="8" t="inlineStr"/>
-      <c r="Y7" s="8" t="inlineStr"/>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="V9" s="9" t="inlineStr">
+        <is>
+          <t>① 진부화·단종·판매부진 재고 식별 절차 확인(회전율 분석 포함) ② 해당 재고 NRV·평가손실 인식 여부 ③ 유효기간·품목허가 변경 등 규제상 판매불가능해진 재고, '유통기한이 없다'는 이유로 평가대상에서 제외된 재고(안료 등 화학제품)가 없는지 확인 ④ 기중 입고만 있고 출고가 없는 품목이 손상평가 대상에서 제외되지 않았는지 확인 ⑤ 품질문제·체화 재고 목록·금액 대사</t>
+        </is>
+      </c>
+      <c r="W9" s="9" t="inlineStr">
+        <is>
+          <t>진부화·단종 재고가 식별·평가되었는가?; 판매부진 재고에 평가손실이 인식되었는가?; 유효기간·품목허가 변경으로 판매불가능해진 재고가 평가대상에서 누락되지 않았는가?; 유통기한이 없다는 이유로 평가대상에서 제외된 재고가 없는가?</t>
+        </is>
+      </c>
+      <c r="X9" s="9" t="inlineStr"/>
+      <c r="Y9" s="9" t="inlineStr"/>
+      <c r="Z9" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 7.16⑵⑶, K-IFRS 1002호 문단28·30</t>
+        </is>
+      </c>
+      <c r="AA9" s="11" t="inlineStr">
+        <is>
+          <t>KSA 501(재고자산 실사입회 — 손상·진부화 징후 관찰)</t>
+        </is>
+      </c>
+      <c r="AB9" s="11" t="inlineStr">
+        <is>
+          <t>FSS2311-08(의약품 제조공장 변경허가로 유효기간 연장 불가에도 평가손실 미인식); KICPA-2024-17(안료는 유통기한이 없다는 이유로 평가충당금 미설정); KICPA-2024-18(입고만 있고 출고 없는 품목을 손상평가 대상에서 제외)</t>
+        </is>
+      </c>
+      <c r="AC9" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 신속처리질의(상품·제품의 감액 회계처리) 문단7·29~33(NRV 추정시 가장 신뢰성 있는 증거 기준)</t>
+        </is>
+      </c>
+      <c r="AD9" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목27(공유)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>L2-03</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>손실부담계약 관련 재고·충당</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>손실부담계약 오류</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 F사</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>저가법 평가·초과 계약물량 충당 구분 오류</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 F사</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>원가보다 낮은 가격으로 공급계약을 체결(손실부담계약)함에 따라 계약이행용 보유 기말재고자산은 저가법 평가손실을, 보유 재고자산 수량을 초과하는 계약물량은 충당부채를 인식하여야 함에도, 재고자산은 취득원가 그대로 계상하고 계약물량 전체에 대해 충당부채를 인식하여 재고자산·충당부채 과대계상</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr"/>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="I10" s="9" t="inlineStr"/>
+      <c r="J10" s="9" t="inlineStr">
         <is>
           <t>손실</t>
         </is>
       </c>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="K10" s="9" t="inlineStr">
         <is>
           <t>손실부담; 충당; 계약; 저가법</t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
+      <c r="L10" s="9" t="inlineStr">
         <is>
           <t>손실부담</t>
         </is>
       </c>
-      <c r="M8" s="8" t="inlineStr">
+      <c r="M10" s="9" t="inlineStr">
         <is>
           <t>저가법; 충당부채</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr"/>
-      <c r="O8" s="8" t="inlineStr">
+      <c r="N10" s="9" t="inlineStr"/>
+      <c r="O10" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호; 1037호</t>
         </is>
       </c>
-      <c r="P8" s="8" t="inlineStr">
-        <is>
-          <t>손실부담계약 재고·충당 인식 검토</t>
-        </is>
-      </c>
-      <c r="Q8" s="8" t="inlineStr">
-        <is>
-          <t>재고 평가와 충당부채 구분 결론 보강</t>
-        </is>
-      </c>
-      <c r="R8" s="8" t="inlineStr">
-        <is>
-          <t>GS-F-L2-03</t>
-        </is>
-      </c>
-      <c r="S8" s="8" t="inlineStr">
+      <c r="P10" s="9" t="inlineStr">
+        <is>
+          <t>손실부담계약 재고·충당 인식 검토를 문서화 바랍니다(보유재고 저가법 평가와 초과계약물량 충당부채를 구분)</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>재고 평가와 충당부채 구분 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R10" s="9" t="inlineStr"/>
+      <c r="S10" s="9" t="inlineStr">
         <is>
           <t>재고자산; 충당부채</t>
         </is>
       </c>
-      <c r="T8" s="8" t="inlineStr">
+      <c r="T10" s="9" t="inlineStr">
         <is>
           <t>재고; 손실부담; 충당</t>
         </is>
       </c>
-      <c r="U8" s="8" t="inlineStr">
+      <c r="U10" s="9" t="inlineStr">
         <is>
           <t>E; FF</t>
         </is>
       </c>
-      <c r="V8" s="8" t="inlineStr">
-        <is>
-          <t>① 손실부담계약 관련 재고·충당부채 구분 확인 ② 저가법 평가와 충당부채 인식 기준 대사 ③ 초과 계약물량·예상손실 반영 결론</t>
-        </is>
-      </c>
-      <c r="W8" s="8" t="inlineStr">
-        <is>
-          <t>재고 평가손실과 손실부담계약 충당이 구분되어 있는가?; 충당부채 인식 요건·금액이 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X8" s="8" t="inlineStr"/>
-      <c r="Y8" s="8" t="inlineStr"/>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="11" t="n">
+      <c r="V10" s="9" t="inlineStr">
+        <is>
+          <t>① 손실부담계약(취소불능 구입계약 포함) 관련 재고·충당부채 구분 확인 ② 보유 재고자산 수량 이내분은 저가법 평가손실로, 초과 계약물량은 K-IFRS1037호에 따른 충당부채로 인식하였는지 확인(둘을 혼동해 재고를 취득원가 그대로 두고 계약물량 전체를 충당부채로 인식하지 않았는지) ③ 충당부채 인식 후 추가 시가하락분이 매출원가에 가산되었는지 확인 ④ 초과 계약물량·예상손실 반영 결론</t>
+        </is>
+      </c>
+      <c r="W10" s="9" t="inlineStr">
+        <is>
+          <t>재고 평가손실과 손실부담계약 충당이 구분되어 있는가?; 충당부채 인식 요건·금액이 문서화되어 있는가?; 충당부채 인식 이후 추가 시가하락분이 매출원가에 가산되었는가?</t>
+        </is>
+      </c>
+      <c r="X10" s="9" t="inlineStr"/>
+      <c r="Y10" s="9" t="inlineStr"/>
+      <c r="Z10" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 7.20, 14.4(충당부채 인식); K-IFRS 1002호 문단31(확정판매계약 초과수량 충당부채는 1037호 회계처리)</t>
+        </is>
+      </c>
+      <c r="AA10" s="11" t="inlineStr">
+        <is>
+          <t>KSA 540(손실부담계약 추정치 감사)</t>
+        </is>
+      </c>
+      <c r="AB10" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 773(재고자산의 취소불능 구입계약 — 품질하자로 잔여물량 매입거부, 상사중재 패소 예상 상황의 충당부채·평가손실 구분 사례)</t>
+        </is>
+      </c>
+      <c r="AC10" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 773(위 인용문: 회피불가능비용이 계약상 효익을 초과할 가능성이 매우 높은 경우 예상손실을 충당부채로 인식, 충당부채 인식 이후 추가 시가하락분은 매출원가 가산)</t>
+        </is>
+      </c>
+      <c r="AD10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>L2-04</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>장기체화·확정판매계약 NRV</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E11" s="9" t="inlineStr">
         <is>
           <t>확정계약 NRV 오류</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>금감원 유의사항 ②</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
         <is>
           <t>확정판매계약 보유 재고에 계약가격 대신 일반 판매가격 적용</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="I11" s="9" t="inlineStr">
         <is>
           <t>확정계약 재고 유의 시</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="J11" s="9" t="inlineStr">
         <is>
           <t>확정</t>
         </is>
       </c>
-      <c r="K9" s="8" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>판매계약; 계약가격; 장기체화; NRV</t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>확정판매; 계약</t>
         </is>
       </c>
-      <c r="M9" s="8" t="inlineStr">
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>계약가격 기초; 계약가격 적용; NRV 산정</t>
         </is>
       </c>
-      <c r="N9" s="8" t="inlineStr">
+      <c r="N11" s="9" t="inlineStr">
         <is>
           <t>일반 판매가만</t>
         </is>
       </c>
-      <c r="O9" s="8" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호</t>
         </is>
       </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>확정판매계약 보유 재고 NRV 산정 검토</t>
-        </is>
-      </c>
-      <c r="Q9" s="8" t="inlineStr">
-        <is>
-          <t>계약가격 기초 NRV 산정 결론 보강</t>
-        </is>
-      </c>
-      <c r="R9" s="8" t="inlineStr">
+      <c r="P11" s="9" t="inlineStr">
+        <is>
+          <t>확정판매계약 보유 재고 NRV 산정 검토를 문서화 바랍니다(초과수량은 일반판매가격 기초)</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>계약가격 기초 NRV 산정 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R11" s="9" t="inlineStr">
         <is>
           <t>GS-F-L2-04</t>
         </is>
       </c>
-      <c r="S9" s="8" t="inlineStr">
+      <c r="S11" s="9" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="T9" s="8" t="inlineStr">
+      <c r="T11" s="9" t="inlineStr">
         <is>
           <t>재고; 확정; 계약; NRV</t>
         </is>
       </c>
-      <c r="U9" s="8" t="inlineStr">
+      <c r="U11" s="9" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="V9" s="8" t="inlineStr">
-        <is>
-          <t>① 확정판매계약 보유 재고 식별 ② NRV 산정 시 계약가격(일반 판매가 아님) 적용 확인 ③ 장기체화 재고 평가 결론</t>
-        </is>
-      </c>
-      <c r="W9" s="8" t="inlineStr">
-        <is>
-          <t>확정판매계약 재고에 계약가격 기초 NRV가 적용되었는가?; 일반 판매가만 사용한 품목이 없는가?</t>
-        </is>
-      </c>
-      <c r="X9" s="8" t="inlineStr"/>
-      <c r="Y9" s="8" t="inlineStr"/>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="V11" s="9" t="inlineStr">
+        <is>
+          <t>① 확정판매계약(주문제작 OEM/ODM 포함) 보유 재고 식별 ② NRV 산정 시 계약가격(일반 판매가 아님) 적용 확인, 계약수량 초과분은 일반판매가격 기초 확인 ③ 발주취소·물량축소가 발생한 경우 일반판매가격으로 재평가되었는지 확인(계약취소시 계약가격 유지 오류 반대유형) ④ 장기체화 재고 평가 결론</t>
+        </is>
+      </c>
+      <c r="W11" s="9" t="inlineStr">
+        <is>
+          <t>확정판매계약 재고에 계약가격 기초 NRV가 적용되었는가?; 일반 판매가만 사용한 품목이 없는가?; 발주취소·물량축소된 확정계약 재고를 일반판매가격으로 재평가하였는가?</t>
+        </is>
+      </c>
+      <c r="X11" s="9" t="inlineStr"/>
+      <c r="Y11" s="9" t="inlineStr"/>
+      <c r="Z11" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 실무지침 실7.7(확정판매계약 이행재고는 계약가격, 초과수량은 일반판매가격), K-IFRS 1002호 문단31</t>
+        </is>
+      </c>
+      <c r="AA11" s="11" t="inlineStr">
+        <is>
+          <t>KSA 540(NRV 추정치 감사)</t>
+        </is>
+      </c>
+      <c r="AB11" s="11" t="inlineStr">
+        <is>
+          <t>FSS2311-09(특정 거래처 주문제작(PCB) 후 발주취소 물량에 평가충당금 미인식)</t>
+        </is>
+      </c>
+      <c r="AC11" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 신속처리질의(상품·제품의 감액 회계처리) 문단31(재수록)</t>
+        </is>
+      </c>
+      <c r="AD11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>L2-05</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>원가 상승·판매가 하락 동시 재평가</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>NRV 미재평가</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>금감원 유의사항 ②</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>원가 상승·판매가 하락이 동시에 발생했으나 평가손실 미인식</t>
         </is>
       </c>
-      <c r="H10" s="9" t="inlineStr">
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="I12" s="9" t="inlineStr">
         <is>
           <t>재고 중요성 이상</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="J12" s="9" t="inlineStr">
         <is>
           <t>원가</t>
         </is>
       </c>
-      <c r="K10" s="8" t="inlineStr">
+      <c r="K12" s="9" t="inlineStr">
         <is>
           <t>상승; 판매가; 하락; NRV; 재평가</t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
+      <c r="L12" s="9" t="inlineStr">
         <is>
           <t>NRV; 원가</t>
         </is>
       </c>
-      <c r="M10" s="8" t="inlineStr">
+      <c r="M12" s="9" t="inlineStr">
         <is>
           <t>평가손실; 순실현; 재측정</t>
         </is>
       </c>
-      <c r="N10" s="8" t="inlineStr">
+      <c r="N12" s="9" t="inlineStr">
         <is>
           <t>원가만 상승; 변동 없음</t>
         </is>
       </c>
-      <c r="O10" s="8" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호</t>
         </is>
       </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>원가·판매가 변동 시 NRV 재평가 검토</t>
-        </is>
-      </c>
-      <c r="Q10" s="8" t="inlineStr">
-        <is>
-          <t>동시 변동 시 평가손실 인식 결론 보강</t>
-        </is>
-      </c>
-      <c r="R10" s="8" t="inlineStr">
+      <c r="P12" s="9" t="inlineStr">
+        <is>
+          <t>원가·판매가 변동 시 NRV 재평가 검토를 문서화 바랍니다(협력사·1차벤더 등 발주처 단가인하 압력과 원가상승이 동시 존재하는 업종 특성 고려)</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>동시 변동 시 평가손실 인식 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R12" s="9" t="inlineStr">
         <is>
           <t>GS-F-L2-05</t>
         </is>
       </c>
-      <c r="S10" s="8" t="inlineStr">
+      <c r="S12" s="9" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="T10" s="8" t="inlineStr">
+      <c r="T12" s="9" t="inlineStr">
         <is>
           <t>재고; 원가; NRV; 평가손실</t>
         </is>
       </c>
-      <c r="U10" s="8" t="inlineStr">
+      <c r="U12" s="9" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="V10" s="8" t="inlineStr">
-        <is>
-          <t>① 원가 상승·판매가 하락 동시 발생 시 NRV 재평가 여부 ② 평가손실 인식 시점·금액 문서화 ③ 당기 변동 요인·결론 기재</t>
-        </is>
-      </c>
-      <c r="W10" s="8" t="inlineStr">
-        <is>
-          <t>원가·판매가 동시 변동 시 NRV가 재평가되었는가?; 평가손실 인식 결론이 있는가?</t>
-        </is>
-      </c>
-      <c r="X10" s="8" t="inlineStr"/>
-      <c r="Y10" s="8" t="inlineStr"/>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="11" t="n">
+      <c r="V12" s="9" t="inlineStr">
+        <is>
+          <t>① 원가 상승·판매가 하락 동시 발생 시 NRV 재평가 여부(발주처 납품단가 인하압력 + 생산차질에 따른 단위당 제조원가 상승 등 업종 특성 고려) ② 평가손실 인식 시점·금액 문서화 ③ 저가법 평가 이력이 다년간 전무한 경우 주석의 저가법 문구가 실제 평가와 일치하는지 확인 ④ 당기 변동 요인·결론 기재</t>
+        </is>
+      </c>
+      <c r="W12" s="9" t="inlineStr">
+        <is>
+          <t>원가·판매가 동시 변동 시 NRV가 재평가되었는가?; 평가손실 인식 결론이 있는가?; 발주처 단가인하압력과 제조원가 상승이 동시에 존재함에도 다년간 저가법 평가 이력이 없지 않은가?</t>
+        </is>
+      </c>
+      <c r="X12" s="9" t="inlineStr"/>
+      <c r="Y12" s="9" t="inlineStr"/>
+      <c r="Z12" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1002호 문단6·9·29, 일반기업회계기준 7.16⑵⑷</t>
+        </is>
+      </c>
+      <c r="AA12" s="11" t="inlineStr">
+        <is>
+          <t>KSA 520(분석적절차 — 매출총이익률 추세 분석)</t>
+        </is>
+      </c>
+      <c r="AB12" s="11" t="inlineStr">
+        <is>
+          <t>FSS1912-1(완성차 협력사, 납품단가 인하(3~5%/년)와 파업으로 인한 제조간접비 상승 동시발생에도 11년간 저가법 미적용, NRV 18.6~40.3% 하락에도 평가손실 0)</t>
+        </is>
+      </c>
+      <c r="AC12" s="11" t="inlineStr"/>
+      <c r="AD12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>L2-06</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>물리적 손상·감모 재고 식별</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>손상 재고 미식별</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>금감원 유의사항 ①</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>파손·유통기한 경과 등 물리적 손상 재고 평가손실 미인식</t>
         </is>
       </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr"/>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr"/>
+      <c r="J13" s="9" t="inlineStr">
         <is>
           <t>손상</t>
         </is>
       </c>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="K13" s="9" t="inlineStr">
         <is>
           <t>파손; 감모; 유통기한; 폐기; 물리적</t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>손상; 식별</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="M13" s="9" t="inlineStr">
         <is>
           <t>평가손실; NRV; 폐기</t>
         </is>
       </c>
-      <c r="N11" s="8" t="inlineStr">
+      <c r="N13" s="9" t="inlineStr">
         <is>
           <t>취득원가 유지</t>
         </is>
       </c>
-      <c r="O11" s="8" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호</t>
         </is>
       </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>물리적 손상 재고 식별·평가손실 검토</t>
-        </is>
-      </c>
-      <c r="Q11" s="8" t="inlineStr">
-        <is>
-          <t>손상 재고 식별·평가 결론 보강</t>
-        </is>
-      </c>
-      <c r="R11" s="8" t="inlineStr">
+      <c r="P13" s="9" t="inlineStr">
+        <is>
+          <t>물리적 손상 재고 식별·평가손실 검토를 문서화 바랍니다(현업 실사결과의 ERP 반영 여부 포함)</t>
+        </is>
+      </c>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>손상 재고 식별·평가 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R13" s="9" t="inlineStr">
         <is>
           <t>GS-F-L2-06</t>
         </is>
       </c>
-      <c r="S11" s="8" t="inlineStr">
+      <c r="S13" s="9" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="T11" s="8" t="inlineStr">
+      <c r="T13" s="9" t="inlineStr">
         <is>
           <t>재고; 손상; 평가손실</t>
         </is>
       </c>
-      <c r="U11" s="8" t="inlineStr">
+      <c r="U13" s="9" t="inlineStr">
         <is>
           <t>E; E100</t>
         </is>
       </c>
-      <c r="V11" s="8" t="inlineStr">
-        <is>
-          <t>① 실사·입회(E100)에서 물리적 손상·유통기한 경과 재고 확인 ② 파손·감모·폐기 대상 식별·평가손실 인식 ③ 손상 재고 목록·금액 문서화</t>
-        </is>
-      </c>
-      <c r="W11" s="8" t="inlineStr">
-        <is>
-          <t>물리적 손상·유통기한 경과 재고가 식별되었는가?; 해당 재고에 평가손실이 인식되었는가?</t>
-        </is>
-      </c>
-      <c r="X11" s="8" t="inlineStr"/>
-      <c r="Y11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="11" t="n">
+      <c r="V13" s="9" t="inlineStr">
+        <is>
+          <t>① 실사·입회(E100)에서 물리적 손상·유통기한 경과 재고 확인 ② 현업 재고실사 결과가 ERP에 반영되는 내부통제 존재 여부 확인(미반영시 감모·평가손실 과소계상 위험) ③ 재고자산 회전율이 지속 하락함에도 개선되지 않았는지 점검 ④ 표본실사만 수행하고 전수실사를 생략하지 않았는지 확인 ⑤ 파손·감모·폐기 대상 식별·평가손실 인식, 손상 재고 목록·금액 문서화</t>
+        </is>
+      </c>
+      <c r="W13" s="9" t="inlineStr">
+        <is>
+          <t>물리적 손상·유통기한 경과 재고가 식별되었는가?; 해당 재고에 평가손실이 인식되었는가?; 현업 실사결과가 ERP에 반영되지 않는 내부통제 미비가 없는가?; 재고자산 회전율이 지속 하락하는데도 개선되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X13" s="9" t="inlineStr"/>
+      <c r="Y13" s="9" t="inlineStr"/>
+      <c r="Z13" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1002호 문단34, 일반기업회계기준 7.16⑴·7.20(감모손실 정상/비정상 구분)</t>
+        </is>
+      </c>
+      <c r="AA13" s="11" t="inlineStr">
+        <is>
+          <t>KSA 501 문단4(재고실사 입회), KSA 530(표본감사 — 전수실사 대체 여부)</t>
+        </is>
+      </c>
+      <c r="AB13" s="11" t="inlineStr">
+        <is>
+          <t>FSS2206-07(현업 재고실사 결과 ERP 미반영 내부통제 미비, 회전율 지속 하락에도 미개선); FSS1912-3(표본실사만 수행, 지정감사인 전수실사 후 장부가 20% 상당 부존재·불량·파손 발견)</t>
+        </is>
+      </c>
+      <c r="AC13" s="11" t="inlineStr"/>
+      <c r="AD13" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목27: 실사조서가 없는 경우, 중요한 타처보관재고 미조회 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>재고자산 평가손실 인식의 적정성</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>L2-07</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>재고 원가 산정(부대비용·정상생산능력)</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>원가 산정 오류</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계오류 예시</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>비정상 생산능력 고정비·부대비용 원가 배분 오류</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계오류 예시</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>비정상 생산능력 고정비·부대비용 원가 배분 오류(물류대행수수료 등을 매출원가에서 판매여부 무관 전액 차감, 신규 외주공정 원가를 대표항목에만 일괄배부)</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>제조업·원가 중요 시</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>원가</t>
         </is>
       </c>
-      <c r="K12" s="8" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
         <is>
           <t>부대비용; 정상생산; 고정비; 배분; 산정</t>
         </is>
       </c>
-      <c r="L12" s="8" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>원가; 산정</t>
         </is>
       </c>
-      <c r="M12" s="8" t="inlineStr">
+      <c r="M14" s="9" t="inlineStr">
         <is>
           <t>부대비용; 정상생산능력</t>
         </is>
       </c>
-      <c r="N12" s="8" t="inlineStr">
+      <c r="N14" s="9" t="inlineStr">
         <is>
           <t>전액 원가</t>
         </is>
       </c>
-      <c r="O12" s="8" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1002호</t>
         </is>
       </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>재고 원가 구성·배분 검토 문서화</t>
-        </is>
-      </c>
-      <c r="Q12" s="8" t="inlineStr">
-        <is>
-          <t>부대비용·정상생산능력 배분 결론 보강</t>
-        </is>
-      </c>
-      <c r="R12" s="8" t="inlineStr">
+      <c r="P14" s="9" t="inlineStr">
+        <is>
+          <t>재고 원가 구성·배분(부대비용·정상생산능력) 검토를 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q14" s="9" t="inlineStr">
+        <is>
+          <t>부대비용·정상생산능력 배분 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R14" s="9" t="inlineStr">
         <is>
           <t>GS-F-L2-07</t>
         </is>
       </c>
-      <c r="S12" s="8" t="inlineStr">
+      <c r="S14" s="9" t="inlineStr">
         <is>
           <t>재고자산</t>
         </is>
       </c>
-      <c r="T12" s="8" t="inlineStr">
+      <c r="T14" s="9" t="inlineStr">
         <is>
           <t>재고; 원가; 부대비용</t>
         </is>
       </c>
-      <c r="U12" s="8" t="inlineStr">
+      <c r="U14" s="9" t="inlineStr">
         <is>
           <t>E; Q</t>
         </is>
       </c>
-      <c r="V12" s="8" t="inlineStr">
-        <is>
-          <t>① 재고 원가 산정(부대비용·정상생산능력·고정비 배분) 검토 ② 비정상 생산능력 고정비 처리 확인 ③ 원가 배분 결론·산식 문서화</t>
-        </is>
-      </c>
-      <c r="W12" s="8" t="inlineStr">
-        <is>
-          <t>부대비용·정상생산능력 기준 원가 배분이 적정한가?; 비정상 생산 시 고정비 처리가 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X12" s="8" t="inlineStr"/>
-      <c r="Y12" s="8" t="inlineStr"/>
-    </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="12" t="n">
+      <c r="V14" s="9" t="inlineStr">
+        <is>
+          <t>① 재고 원가 산정(부대비용·정상생산능력·고정비 배분) 검토 ② 비정상 생산능력(유휴설비 등) 고정비를 원가에 비정상적으로 가산하지 않았는지 확인 ③ 물류대행수수료·리베이트 등 매입할인 성격 금액을 판매여부와 무관하게 매출원가에서 전액 차감(미판매분은 재고원가에서 차감해야 함)하지 않았는지 확인 ④ 신규 외주공정 발생원가가 대표항목에만 일괄배부되지 않고 세부 품목별로 배분되는지 확인 ⑤ 원가 배분 결론·산식 문서화</t>
+        </is>
+      </c>
+      <c r="W14" s="9" t="inlineStr">
+        <is>
+          <t>부대비용·정상생산능력 기준 원가 배분이 적정한가?; 비정상 생산 시 고정비 처리가 문서화되어 있는가?; 매입 관련 수수료·리베이트가 매출원가에서 판매여부와 무관하게 전액 차감되고 있지 않은가?; 신규 공정 발생원가가 세부 품목별로 적절히 배분되는가?</t>
+        </is>
+      </c>
+      <c r="X14" s="9" t="inlineStr"/>
+      <c r="Y14" s="9" t="inlineStr"/>
+      <c r="Z14" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 7.6(매입할인 차감), 7.8(정상조업도 — 비정상적으로 낮은 조업도·유휴설비 배부액 증가 금지), 7.9(공통원가 배분), 실무지침 실7.11(소비세 제외)</t>
+        </is>
+      </c>
+      <c r="AA14" s="11" t="inlineStr">
+        <is>
+          <t>KSA 520(분석적절차 — 원가율 추세)</t>
+        </is>
+      </c>
+      <c r="AB14" s="11" t="inlineStr">
+        <is>
+          <t>FSS2512-07(신규 외주공정 원가를 기타 계정으로 분류 후 전액 기말재고로 배부, 원재료를 대표항목에만 배부); FSS2405-08(물류대행수수료 등을 매출원가에서 전액 차감, 매입할인 성격이므로 미판매분은 재고원가에서 차감해야 함)</t>
+        </is>
+      </c>
+      <c r="AC14" s="11" t="inlineStr"/>
+      <c r="AD14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>재고자산 평가손실 인식의 적정성</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>L2-08</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관재고(제3자 보관재고) 실재성 확인</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관재고 조회 미실시</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>금감원·한공회 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>하청업체·물류창고 등 제3자 보관재고에 대해 감사인이 직접 조회서를 발송·회수하지 않고 회사를 통해 수발신하거나, 보관증 위조·비정상적 증가에도 직접조회를 생략</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>검토누락</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관재고 유의적인 경우</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관</t>
+        </is>
+      </c>
+      <c r="K15" s="9" t="inlineStr">
+        <is>
+          <t>제3자보관; 위탁재고; 조회서; 보세창고</t>
+        </is>
+      </c>
+      <c r="L15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관재고 조회</t>
+        </is>
+      </c>
+      <c r="M15" s="9" t="inlineStr">
+        <is>
+          <t>감사인 직접 발송·회수; 독립적 조회</t>
+        </is>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
+          <t>회사경유 발송; 보관증 위조</t>
+        </is>
+      </c>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>회계감사기준서 505; 501</t>
+        </is>
+      </c>
+      <c r="P15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관재고에 대한 감사인 직접 조회(발송·회수 통제) 절차를 수행·문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>조회처 독립성 확인 및 실재성 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R15" s="9" t="inlineStr"/>
+      <c r="S15" s="9" t="inlineStr">
+        <is>
+          <t>재고자산</t>
+        </is>
+      </c>
+      <c r="T15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관; 위탁재고; 보세창고</t>
+        </is>
+      </c>
+      <c r="U15" s="9" t="inlineStr">
+        <is>
+          <t>E; CS</t>
+        </is>
+      </c>
+      <c r="V15" s="9" t="inlineStr">
+        <is>
+          <t>① 타처보관(제3자보관) 재고자산의 중요성 여부 확인 ② 감사인이 조회서를 직접 발송·회수하였는지(회사를 통한 수발신이 아닌지) 확인 ③ 조회처(하청업체·물류창고 등)의 독립성 및 보관증 진위 확인 ④ 타처보관재고가 비정상적으로 증가(실제 대비 수배 등)하였음에도 직접조회를 생략하지 않았는지 점검</t>
+        </is>
+      </c>
+      <c r="W15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관 재고자산에 대해 감사인이 직접 발송·회수하였는가?; 조회처의 독립성이 확인되었는가?; 타처보관재고가 비정상적으로 증가하였음에도 직접조회를 생략하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X15" s="9" t="inlineStr"/>
+      <c r="Y15" s="9" t="inlineStr">
+        <is>
+          <t>타처보관재고가 없는 경우</t>
+        </is>
+      </c>
+      <c r="Z15" s="11" t="inlineStr"/>
+      <c r="AA15" s="11" t="inlineStr">
+        <is>
+          <t>KSA 505 문단7(조회서 발송·회수 통제 유지), KSA 501 문단A1·A2·A4</t>
+        </is>
+      </c>
+      <c r="AB15" s="11" t="inlineStr">
+        <is>
+          <t>FSS2512-06(하청 보관처에 허위회신 요구); KICPA-2021-04(타처보관재고 실제의 4배 이상 비정상 증가에도 직접조회 생략); 구 FSS 사례집(제3자 직접조회 없이 회사경유 조회서만 확인, 보관증 위조)</t>
+        </is>
+      </c>
+      <c r="AC15" s="11" t="inlineStr"/>
+      <c r="AD15" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목27: 중요한 타처보관재고 미조회, 타처보관재고조회서상 차이내역 미소명 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>재고자산 평가손실 인식의 적정성</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>L2-09</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>재고자산 실사입회의 완전성</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>실사입회 누락·부실</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>금감원·한공회 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>입회시점과 실사시점이 상이하여 실질적으로 입회가 이루어지지 않거나, 회사가 제공한 실사목록만으로 입회를 대체, 매장·창고 일부를 실사하지 않음</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>검토누락</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr"/>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>실사입회</t>
+        </is>
+      </c>
+      <c r="K16" s="9" t="inlineStr">
+        <is>
+          <t>입회; 실사시점; 표본추출; 창고</t>
+        </is>
+      </c>
+      <c r="L16" s="9" t="inlineStr">
+        <is>
+          <t>실사입회 조서</t>
+        </is>
+      </c>
+      <c r="M16" s="9" t="inlineStr">
+        <is>
+          <t>입회 수행; 독립적 실사목록; 표본추출근거</t>
+        </is>
+      </c>
+      <c r="N16" s="9" t="inlineStr">
+        <is>
+          <t>회사제공목록만; 입회시점 상이</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
+        <is>
+          <t>회계감사기준서 501; 530</t>
+        </is>
+      </c>
+      <c r="P16" s="9" t="inlineStr">
+        <is>
+          <t>재고자산 실사입회(입회시점·표본추출·매장별 커버리지)를 검토·문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>실사입회 커버리지 및 재고특성 고려 여부 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R16" s="9" t="inlineStr"/>
+      <c r="S16" s="9" t="inlineStr">
+        <is>
+          <t>재고자산</t>
+        </is>
+      </c>
+      <c r="T16" s="9" t="inlineStr">
+        <is>
+          <t>실사; 입회; 창고; 매장</t>
+        </is>
+      </c>
+      <c r="U16" s="9" t="inlineStr">
+        <is>
+          <t>E; E100</t>
+        </is>
+      </c>
+      <c r="V16" s="9" t="inlineStr">
+        <is>
+          <t>① 실사입회 시점과 재고 기준시점(결산일)의 상이 여부 확인(상이한 경우 조정절차 필요) ② 회사가 제공한 실사목록을 그대로 사용하지 않고 감사인이 독자적으로 표본을 추출하였는지 확인 ③ 매장·창고·물류센터 등 보관장소별 실사 커버리지(일부 매장 미실사 여부) 확인 ④ 재고 특성(스크랩·야적재고 등)을 고려한 실사방법을 사용하였는지 확인</t>
+        </is>
+      </c>
+      <c r="W16" s="9" t="inlineStr">
+        <is>
+          <t>실사입회 시점과 재고 기준시점이 상이하지 않은가?; 회사가 제공한 실사목록만으로 입회를 대체하지 않았는가?; 매장·창고 일부가 실사에서 누락되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X16" s="9" t="inlineStr"/>
+      <c r="Y16" s="9" t="inlineStr"/>
+      <c r="Z16" s="11" t="inlineStr"/>
+      <c r="AA16" s="11" t="inlineStr">
+        <is>
+          <t>KSA 501 문단4·A1~A4(재고실사 입회), KSA 530 문단A5(표본감사)</t>
+        </is>
+      </c>
+      <c r="AB16" s="11" t="inlineStr">
+        <is>
+          <t>FSS2008-13(입회시점과 실사시점이 상이하여 실질적 미입회); FSS2409-07(회사제공 실사목록만으로 입회); KICPA-2024-47(매장보관재고 실사입회 누락, 위험평가절차·통제테스트 생략); 구 FSS 사례집(원부자재 31% 실사 누락, 매장 다수 미실사)</t>
+        </is>
+      </c>
+      <c r="AC16" s="11" t="inlineStr"/>
+      <c r="AD16" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목27: 실사조서가 없는 경우 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>투자부동산 회계처리</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>L3-01</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>투자부동산·자가사용 분류</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>계정분류 오류</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 G사</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>임대 부분을 유형자산으로 오분류</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 G사</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>자가사용 및 임대수익 목적으로 부동산을 취득하여 일부는 사무실로 사용하고 나머지는 제3자에게 사무실·창고 용도로 임대하였음에도, 제3자 임대 부분을 투자부동산이 아닌 유형자산으로 잘못 분류하여 투자부동산 과소계상</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr"/>
-      <c r="J13" s="8" t="inlineStr">
+      <c r="I17" s="9" t="inlineStr"/>
+      <c r="J17" s="9" t="inlineStr">
         <is>
           <t>투자부동산</t>
         </is>
       </c>
-      <c r="K13" s="8" t="inlineStr">
+      <c r="K17" s="9" t="inlineStr">
         <is>
           <t>분류; 임대; 자가사용; 유형자산</t>
         </is>
       </c>
-      <c r="L13" s="8" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
         <is>
           <t>분류</t>
         </is>
       </c>
-      <c r="M13" s="8" t="inlineStr">
+      <c r="M17" s="9" t="inlineStr">
         <is>
           <t>투자부동산; 임대수익</t>
         </is>
       </c>
-      <c r="N13" s="8" t="inlineStr">
+      <c r="N17" s="9" t="inlineStr">
         <is>
           <t>유형자산만</t>
         </is>
       </c>
-      <c r="O13" s="8" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1040호</t>
         </is>
       </c>
-      <c r="P13" s="8" t="inlineStr">
-        <is>
-          <t>보유목적별 분류 검토·결론 문서화</t>
-        </is>
-      </c>
-      <c r="Q13" s="8" t="inlineStr">
-        <is>
-          <t>임대·자가사용 구분 결론 보강</t>
-        </is>
-      </c>
-      <c r="R13" s="8" t="inlineStr"/>
-      <c r="S13" s="8" t="inlineStr">
+      <c r="P17" s="9" t="inlineStr">
+        <is>
+          <t>보유목적별(임대·자가사용·처분) 분류 검토·결론을 문서화 바랍니다(미분양 후 장기임대전환 등 용도변경 포함)</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>임대·자가사용 구분 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R17" s="9" t="inlineStr"/>
+      <c r="S17" s="9" t="inlineStr">
         <is>
           <t>투자부동산; 유형자산</t>
         </is>
       </c>
-      <c r="T13" s="8" t="inlineStr">
+      <c r="T17" s="9" t="inlineStr">
         <is>
           <t>투자부동산; 임대; 공정가치</t>
         </is>
       </c>
-      <c r="U13" s="8" t="inlineStr">
+      <c r="U17" s="9" t="inlineStr">
         <is>
           <t>F; G</t>
         </is>
       </c>
-      <c r="V13" s="8" t="inlineStr">
-        <is>
-          <t>① F Lead에서 보유목적(임대·자가사용·처분)별 분류 확인 ② 임대 부분 투자부동산 vs 유형자산 구분 ③ 분류 변경·재분류 결론 문서화</t>
-        </is>
-      </c>
-      <c r="W13" s="8" t="inlineStr">
-        <is>
-          <t>임대·자가사용 목적에 따른 분류가 적정한가?; 투자부동산·유형자산 오분류가 없는가?</t>
-        </is>
-      </c>
-      <c r="X13" s="8" t="inlineStr"/>
-      <c r="Y13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="12" t="n">
+      <c r="V17" s="9" t="inlineStr">
+        <is>
+          <t>① F Lead에서 보유목적(임대·자가사용·처분)별 분류 확인 ② 임대 부분 투자부동산 vs 유형자산 구분, 부분임대시 분리매각 가능 여부(불가시 자가사용 부분이 경미한 경우에만 전체를 투자부동산으로 분류) 확인 ③ 미분양 재고자산을 장기임대로 전환하였음에도 재고자산으로 계속 분류하지 않았는지, 경영진의 용도변경 의도 표명만으로 계정대체하지 않았는지(객관적 증거 필요) 확인 ④ 분류·재분류 결론 문서화</t>
+        </is>
+      </c>
+      <c r="W17" s="9" t="inlineStr">
+        <is>
+          <t>임대·자가사용 목적에 따른 분류가 적정한가?; 투자부동산·유형자산 오분류가 없는가?; 미분양되어 장기 임대 중인 자산을 재고자산으로 계속 분류하고 있지 않은가?; 경영진의 용도변경 의도 표명만을 근거로 계정대체하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X17" s="9" t="inlineStr"/>
+      <c r="Y17" s="9" t="inlineStr"/>
+      <c r="Z17" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호 문단5·7-15(정의·분류원칙), 문단10(부분임대 안분·경미기준), 문단57·BC23-29(계정대체는 용도변경의 증거가 있는 경우만); 일반기업회계기준 10.3(투자부동산도 유형자산장 준용, 표시과목만 투자자산)</t>
+        </is>
+      </c>
+      <c r="AA17" s="11" t="inlineStr">
+        <is>
+          <t>KSA 500 문단8(전문가 정보 이용시 평가), KSA 315(자산분류 관련 통제 이해)</t>
+        </is>
+      </c>
+      <c r="AB17" s="11" t="inlineStr">
+        <is>
+          <t>KICPA-2021-14(분양사업을 4년 임대 후 분양으로 변경했음에도 재고자산 계속 계상, 투자부동산 미대체); KICPA-2020-21·2020-22·2022-21(미분양 상가·공동주택 장기임대에도 재고자산 유지, 감가상각 누락)</t>
+        </is>
+      </c>
+      <c r="AC17" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 1780(투자부동산·유형자산 분류, 골프장 임대 사례); 1924(공용면적 안분계산); 1786(부분임대 부동산의 별도재무제표 분류 — 분리매각 의도 없음은 제약사유 아님); 1979(공장 일부 하청업체 임대시 투자부동산 여부); 1399(부동산임대업자의 운용리스 제공 부동산 분류)</t>
+        </is>
+      </c>
+      <c r="AD17" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목28 유형자산/투자부동산(G,F): 분류(취득원가 결정, 유형자산 또는 투자부동산으로의 분류 적정성) 검토내역 부실기재 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>투자부동산 회계처리</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>L3-02</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>공정가치모형 매기 평가</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>공정가치 미평가</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 H사</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>공정가치모형 선택 후 일부 연도 평가 생략</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 H사</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>임대수익 및 시세차익을 목적으로 보유하는 부동산을 투자부동산으로 분류하고 공정가치모형을 선택하여 x1년말 기준 공정가치 평가를 실시하였으나, x2년과 x3년에는 공정가치 변동이 크지 않다고 판단하여 평가를 실시하지 않아 당기순이익 과소계상</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr"/>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="I18" s="9" t="inlineStr"/>
+      <c r="J18" s="9" t="inlineStr">
         <is>
           <t>공정가치</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="K18" s="9" t="inlineStr">
         <is>
           <t>평가; 감정; DCF; 매기</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr">
         <is>
           <t>공정가치</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>평가 실시; 감정; 공정가치</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="N18" s="9" t="inlineStr">
         <is>
           <t>평가 생략; 변동 없음</t>
         </is>
       </c>
-      <c r="O14" s="8" t="inlineStr">
+      <c r="O18" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1040호</t>
         </is>
       </c>
-      <c r="P14" s="8" t="inlineStr">
-        <is>
-          <t>공정가치모형 매기 평가 절차·결과 문서화</t>
-        </is>
-      </c>
-      <c r="Q14" s="8" t="inlineStr">
-        <is>
-          <t>당기 공정가치 평가 수행·결론 보강</t>
-        </is>
-      </c>
-      <c r="R14" s="8" t="inlineStr"/>
-      <c r="S14" s="8" t="inlineStr">
+      <c r="P18" s="9" t="inlineStr">
+        <is>
+          <t>공정가치모형 매기 평가 절차·결과를 문서화 바랍니다(K-GAAP 재평가모형과 K-IFRS 공정가치모형의 회계처리 차이 구분 포함)</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
+        <is>
+          <t>당기 공정가치 평가 수행·결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R18" s="9" t="inlineStr"/>
+      <c r="S18" s="9" t="inlineStr">
         <is>
           <t>투자부동산</t>
         </is>
       </c>
-      <c r="T14" s="8" t="inlineStr">
+      <c r="T18" s="9" t="inlineStr">
         <is>
           <t>투자부동산; 공정가치</t>
         </is>
       </c>
-      <c r="U14" s="8" t="inlineStr">
+      <c r="U18" s="9" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="V14" s="8" t="inlineStr">
-        <is>
-          <t>① 공정가치모형 선택 시 당기 평가 수행 여부 ② 감정·DCF 등 평가 방법·가정·결과 문서화 ③ 변동손익 인식 결론</t>
-        </is>
-      </c>
-      <c r="W14" s="8" t="inlineStr">
-        <is>
-          <t>공정가치모형 적용 시 당기 평가가 수행되었는가?; 평가 방법·가정·결론이 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X14" s="8" t="inlineStr"/>
-      <c r="Y14" s="8" t="inlineStr"/>
-    </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="12" t="n">
+      <c r="V18" s="9" t="inlineStr">
+        <is>
+          <t>① 공정가치모형 선택 시 당기 평가 수행 여부(변동이 크지 않다는 판단만으로 생략하지 않았는지) ② 감정·DCF 등 평가 방법·가정·결과 문서화 ③ 재평가이익 산정시 총장부금액이 아닌 순장부금액 기준으로 계산되었는지 확인 ④ K-GAAP 적용회사가 '공정가치모형' 용어를 사용하면서 실제로는 감가상각 생략·손익 당기인식 등 IFRS식 회계처리를 잘못 차용하지 않았는지 확인(K-GAAP은 재평가모형만 존재, OCI 인식·감가상각 계속이 원칙) ⑤ 변동손익 인식 결론</t>
+        </is>
+      </c>
+      <c r="W18" s="9" t="inlineStr">
+        <is>
+          <t>공정가치모형 적용 시 당기 평가가 수행되었는가?; 평가 방법·가정·결론이 문서화되어 있는가?; 재평가이익을 순장부금액이 아닌 총장부금액 기준으로 산정하지 않았는가?; K-GAAP 재평가모형 적용자산에 대해 감가상각을 생략하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X18" s="9" t="inlineStr"/>
+      <c r="Y18" s="9" t="inlineStr"/>
+      <c r="Z18" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호 문단33(매기 공정가치 적용)·문단35(당기손익); 일반기업회계기준 10.22·10.24(K-GAAP 재평가모형 — OCI 인식·감가상각 계속, IFRS 공정가치모형과 상이)</t>
+        </is>
+      </c>
+      <c r="AA18" s="11" t="inlineStr">
+        <is>
+          <t>KSA 620 문단9·12(감사인이 이용하는 전문가의 역량·객관성 평가)</t>
+        </is>
+      </c>
+      <c r="AB18" s="11" t="inlineStr">
+        <is>
+          <t>KICPA-2022-14(재평가모형 선택 후 공정가치가 크게 상승했음에도 재평가 미실시); KICPA-2022-15(재평가이익 산정시 총장부금액 기준 오류)</t>
+        </is>
+      </c>
+      <c r="AC18" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 1792(공정가치모형 적용시 감가상각 불요, 손익은 당기손익); 1678(원가→공정가치 모형 변경은 허용되나 역방향은 사실상 불허); 2085(원가모형 적용 투자부동산의 손상검사는 원칙적으로 개별자산별 수행)</t>
+        </is>
+      </c>
+      <c r="AD18" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목28(공유)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>투자부동산 회계처리</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>L3-03</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>투자부동산 주석 공시</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E19" s="9" t="inlineStr">
         <is>
           <t>주석 미흡</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 I사</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>원가모형 적용 시 공정가치 주석 누락</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 I사</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>임대중인 본사사옥 일부를 투자부동산으로 분류하여 원가모형을 적용하였는데, 원가모형 적용시 공정가치를 주석으로 공시하여야 하나 관련 공시를 소홀히 함</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr"/>
-      <c r="J15" s="8" t="inlineStr">
+      <c r="I19" s="9" t="inlineStr"/>
+      <c r="J19" s="9" t="inlineStr">
         <is>
           <t>주석</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr">
+      <c r="K19" s="9" t="inlineStr">
         <is>
           <t>공시; 공정가치; 장부금액</t>
         </is>
       </c>
-      <c r="L15" s="8" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>주석; 공시</t>
         </is>
       </c>
-      <c r="M15" s="8" t="inlineStr">
+      <c r="M19" s="9" t="inlineStr">
         <is>
           <t>공정가치; 변동</t>
         </is>
       </c>
-      <c r="N15" s="8" t="inlineStr">
+      <c r="N19" s="9" t="inlineStr">
         <is>
           <t>공시 없음</t>
         </is>
       </c>
-      <c r="O15" s="8" t="inlineStr">
+      <c r="O19" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1040호</t>
         </is>
       </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>투자부동산 주석 공시 항목 검토</t>
-        </is>
-      </c>
-      <c r="Q15" s="8" t="inlineStr">
-        <is>
-          <t>공정가치·변동 내역 공시 보강</t>
-        </is>
-      </c>
-      <c r="R15" s="8" t="inlineStr"/>
-      <c r="S15" s="8" t="inlineStr">
+      <c r="P19" s="9" t="inlineStr">
+        <is>
+          <t>투자부동산 주석 공시 항목(공정가치·변동·장부금액, 독립평가인 활용여부, 권리제한사항 등)을 검토 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>공정가치·변동 내역 공시를 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R19" s="9" t="inlineStr"/>
+      <c r="S19" s="9" t="inlineStr">
         <is>
           <t>투자부동산</t>
         </is>
       </c>
-      <c r="T15" s="8" t="inlineStr">
+      <c r="T19" s="9" t="inlineStr">
         <is>
           <t>투자부동산; 주석; 공시</t>
         </is>
       </c>
-      <c r="U15" s="8" t="inlineStr">
+      <c r="U19" s="9" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="V15" s="8" t="inlineStr">
-        <is>
-          <t>① 투자부동산 주석 공시 항목(공정가치·변동·장부금액) 확인 ② 원가모형 적용 시 공정가치 주석 포함 여부 ③ 공시 누락·불충분 항목 식별</t>
-        </is>
-      </c>
-      <c r="W15" s="8" t="inlineStr">
-        <is>
-          <t>투자부동산 주석 공시가 충분한가?; 원가모형 적용 시 공정가치 주석이 있는가?</t>
-        </is>
-      </c>
-      <c r="X15" s="8" t="inlineStr"/>
-      <c r="Y15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="13" t="n">
+      <c r="V19" s="9" t="inlineStr">
+        <is>
+          <t>① 투자부동산 주석 공시 항목(공정가치·변동·장부금액) 확인 ② 원가모형 적용 시 공정가치 주석 포함 여부(공시 목적상 공정가치 측정 필요) 확인 ③ 공정가치가 독립된 평가인의 평가에 근거한 정도 및 미실시시 그 사실 공시 여부 확인 ④ 담보·신탁 제공, 가처분·가압류 등 권리제한 사실이 등기부등본 대사를 통해 주석에 반영되었는지 확인 ⑤ 공시 누락·불충분 항목 식별</t>
+        </is>
+      </c>
+      <c r="W19" s="9" t="inlineStr">
+        <is>
+          <t>투자부동산 주석 공시가 충분한가?; 원가모형 적용 시 공정가치 주석이 있는가?; 공정가치가 독립평가인의 평가에 근거한 정도가 공시되었는가?; 담보·신탁·가처분 등 권리제한 사실이 등기부등본 대사로 확인·공시되었는가?</t>
+        </is>
+      </c>
+      <c r="X19" s="9" t="inlineStr"/>
+      <c r="Y19" s="9" t="inlineStr"/>
+      <c r="Z19" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호 문단75⑸(독립평가인 평가 근거 정도), 문단79(원가모형 공정가치 공시의무), 문단32; 일반기업회계기준 10.48(투자자산인 투자부동산 토지 공시지가 추가 기재)</t>
+        </is>
+      </c>
+      <c r="AA19" s="11" t="inlineStr">
+        <is>
+          <t>KSA 500 문단8, KSA 620 문단9·12(감정평가사 활용 감사절차), KSA 505(외부조회 — 등기부등본·금융기관조회서 대사)</t>
+        </is>
+      </c>
+      <c r="AB19" s="11" t="inlineStr">
+        <is>
+          <t>FSS2008-28(합병취득 유형자산 감가상각누계액 합산 누락으로 주석 과소기재); FSS2008-21(비업무용부동산 손상평가시 토지·건물 일괄평가); FSS2008-30(담보제공 자산 주석 미기재·과소기재, 등기부등본 대사 소홀); FSS2008-29(가처분결정에 따른 권리제한 사실 미공시)</t>
+        </is>
+      </c>
+      <c r="AC19" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 1792, 2085(공유)</t>
+        </is>
+      </c>
+      <c r="AD19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>투자부동산 회계처리</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>L3-04</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>권리관계 확인(등기부등본 대사)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>권리제한사실 미확인</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>금감원 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>대출 상환 후에도 담보제공 사실을 주석에 과소·잘못 기재, 신탁등기 말소 후에도 계속 담보제공된 것으로 오기재, 가처분·가압류 등 권리제한 사실 미공시</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>검토누락</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr"/>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>등기부등본</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>담보제공; 신탁등기; 가압류; 가처분; 근저당</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>등기부등본 대사</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>등기부등본 대사 수행; 권리제한 확인</t>
+        </is>
+      </c>
+      <c r="N20" s="9" t="inlineStr">
+        <is>
+          <t>등기부등본 미확인</t>
+        </is>
+      </c>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호; 일반기업회계기준 제10장</t>
+        </is>
+      </c>
+      <c r="P20" s="9" t="inlineStr">
+        <is>
+          <t>담보·신탁 제공 부동산에 대한 등기부등본 대사 절차를 수행하고, 가처분·가압류 등 권리제한 사실을 확인·문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>금융기관조회서·은행연합회 자료와의 대사 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R20" s="9" t="inlineStr"/>
+      <c r="S20" s="9" t="inlineStr">
+        <is>
+          <t>투자부동산; 유형자산</t>
+        </is>
+      </c>
+      <c r="T20" s="9" t="inlineStr">
+        <is>
+          <t>투자부동산; 담보; 등기</t>
+        </is>
+      </c>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>F; G; CL</t>
+        </is>
+      </c>
+      <c r="V20" s="9" t="inlineStr">
+        <is>
+          <t>① 담보·신탁 제공 부동산의 등기부등본을 결산일 기준으로 열람·대사 ② 대출 상환·신탁등기 말소 후에도 담보제공 사실이 잘못 유지 기재되지 않았는지 확인 ③ 가압류·가처분 등 권리제한 사실이 있는지 확인하고 주석 반영 여부 점검 ④ 금융기관조회서·은행연합회 자료와 교차 대사</t>
+        </is>
+      </c>
+      <c r="W20" s="9" t="inlineStr">
+        <is>
+          <t>담보·신탁 제공 부동산에 대한 등기부등본 대사 절차가 수행되었는가?; 가처분·가압류 등 권리제한 사실이 확인·공시되었는가?; 상환된 대출의 담보제공 사실이 잘못 유지 기재되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X20" s="9" t="inlineStr"/>
+      <c r="Y20" s="9" t="inlineStr">
+        <is>
+          <t>담보·신탁 제공된 부동산이 없는 경우</t>
+        </is>
+      </c>
+      <c r="Z20" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호 문단75⑺, 일반기업회계기준 10.48⑶</t>
+        </is>
+      </c>
+      <c r="AA20" s="11" t="inlineStr">
+        <is>
+          <t>KSA 505(외부조회 — 금융기관조회서)</t>
+        </is>
+      </c>
+      <c r="AB20" s="11" t="inlineStr">
+        <is>
+          <t>FSS2008-30(대출 상환 후에도 담보제공 사실 과소기재, 신탁등기 말소 후 계속 담보제공으로 오기재); FSS2008-29(가처분결정에 따른 권리제한 사실 미공시)</t>
+        </is>
+      </c>
+      <c r="AC20" s="11" t="inlineStr"/>
+      <c r="AD20" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목28: 중요한 자산에 대한 실재성 및 권리관계(등기부등본, 취득test 포함) 검토내역 누락 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>투자부동산 회계처리</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>L3-05</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>독립평가인 자격 및 감정평가 활용 적정성</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>평가인 자격·독립성 미확인</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>금감원 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>공정가치 측정을 위한 감정평가서의 평가인 자격·독립성·유사부동산 평가경험을 확인하지 않고 그대로 이용, 평가기준일과 결산일 간 시장상황 변동을 검토하지 않음</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>결론미비</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr"/>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>감정평가</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>평가기준일; 독립성확인; 평가경험; 재평가주기</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>평가인 적격성 확인</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>평가인 자격 확인; 독립성 확인; 평가기준일 검토</t>
+        </is>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>자격확인 없음</t>
+        </is>
+      </c>
+      <c r="O21" s="9" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호</t>
+        </is>
+      </c>
+      <c r="P21" s="9" t="inlineStr">
+        <is>
+          <t>감정평가서 평가인의 자격요건·독립성·유사부동산 평가경험 확인절차 및 평가기준일과 결산일 간 시장상황 변동 검토를 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>평가인 적격성·평가기준일 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R21" s="9" t="inlineStr"/>
+      <c r="S21" s="9" t="inlineStr">
+        <is>
+          <t>투자부동산</t>
+        </is>
+      </c>
+      <c r="T21" s="9" t="inlineStr">
+        <is>
+          <t>투자부동산; 감정평가; 공정가치</t>
+        </is>
+      </c>
+      <c r="U21" s="9" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="V21" s="9" t="inlineStr">
+        <is>
+          <t>① 감정평가서 평가기준일과 결산일 간 시장상황 변동 여부 검토 ② 평가인의 자격요건·독립성·평가대상 지역 유사부동산 평가경험 확인절차 수행 여부 ③ 재평가주기(3년/5년 등)의 합리성 검토 ④ 감사인측 전문가 활용시 KSA620에 따른 역량·객관성 평가 수행 여부</t>
+        </is>
+      </c>
+      <c r="W21" s="9" t="inlineStr">
+        <is>
+          <t>감정평가서 평가기준일과 결산일 간 시장상황 변동을 검토하였는가?; 평가인의 자격요건·독립성·유사부동산 평가경험을 확인하였는가?</t>
+        </is>
+      </c>
+      <c r="X21" s="9" t="inlineStr"/>
+      <c r="Y21" s="9" t="inlineStr">
+        <is>
+          <t>외부평가인을 이용하지 않는 경우</t>
+        </is>
+      </c>
+      <c r="Z21" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1040호 문단32·75⑸; 일반기업회계기준 10.19·10.25</t>
+        </is>
+      </c>
+      <c r="AA21" s="11" t="inlineStr">
+        <is>
+          <t>KSA 620 문단9·12(감사인측 전문가의 역량·능력·객관성 및 업무 적정성 평가)</t>
+        </is>
+      </c>
+      <c r="AB21" s="11" t="inlineStr"/>
+      <c r="AC21" s="11" t="inlineStr"/>
+      <c r="AD21" s="11" t="inlineStr"/>
+    </row>
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>충당부채의 인식·측정과 우발부채 공시</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>L4-01</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>보증·손실부담 충당부채</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>보증충당 미인식</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 J사</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>보증발전량 미달에도 낙관적 예상으로 충당 미계상</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 J사</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>태양광 발전사업 건설공사 도급계약서상 보증발전량 미달시 손실보전 의무가 있어 충당부채 인식 사유에 해당하였으나, 성능 개선을 통해 잔여기간 동안 보증발전량을 달성할 수 있다는 낙관적 예상을 근거로 보증충당부채를 적립하지 않음</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
+      <c r="I22" s="9" t="inlineStr">
         <is>
           <t>보증·손실부담 유의 시</t>
         </is>
       </c>
-      <c r="J16" s="8" t="inlineStr">
+      <c r="J22" s="9" t="inlineStr">
         <is>
           <t>충당</t>
         </is>
       </c>
-      <c r="K16" s="8" t="inlineStr">
+      <c r="K22" s="9" t="inlineStr">
         <is>
           <t>보증; 손실부담; 최선의 추정</t>
         </is>
       </c>
-      <c r="L16" s="8" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr">
         <is>
           <t>충당</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr">
+      <c r="M22" s="9" t="inlineStr">
         <is>
           <t>보증; 충당부채; 인식</t>
         </is>
       </c>
-      <c r="N16" s="8" t="inlineStr">
+      <c r="N22" s="9" t="inlineStr">
         <is>
           <t>충당 없음; 낙관적</t>
         </is>
       </c>
-      <c r="O16" s="8" t="inlineStr">
+      <c r="O22" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1037호</t>
         </is>
       </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>보증·손실부담 충당 인식요건 검토·결론</t>
-        </is>
-      </c>
-      <c r="Q16" s="8" t="inlineStr">
-        <is>
-          <t>충당부채 인식·측정 결론 보강</t>
-        </is>
-      </c>
-      <c r="R16" s="8" t="inlineStr"/>
-      <c r="S16" s="8" t="inlineStr">
+      <c r="P22" s="9" t="inlineStr">
+        <is>
+          <t>보증·손실부담 충당 인식요건 검토·결론을 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>충당부채 인식·측정(기댓값·최선의 추정치) 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R22" s="9" t="inlineStr"/>
+      <c r="S22" s="9" t="inlineStr">
         <is>
           <t>충당부채; 우발부채·약정</t>
         </is>
       </c>
-      <c r="T16" s="8" t="inlineStr">
+      <c r="T22" s="9" t="inlineStr">
         <is>
           <t>충당; 우발; 보증</t>
         </is>
       </c>
-      <c r="U16" s="8" t="inlineStr">
+      <c r="U22" s="9" t="inlineStr">
         <is>
           <t>FF; CL</t>
         </is>
       </c>
-      <c r="V16" s="8" t="inlineStr">
-        <is>
-          <t>① FF·CL에서 보증·손실부담 관련 충당 인식요건 검토 ② 최선의 추정치·현재가치 측정 문서화 ③ 낙관적 가정만으로 충당 미계상 여부 점검</t>
-        </is>
-      </c>
-      <c r="W16" s="8" t="inlineStr">
-        <is>
-          <t>보증·손실부담 충당 인식요건이 충족되는가?; 충당부채 측정·결론이 문서화되어 있는가?</t>
-        </is>
-      </c>
-      <c r="X16" s="8" t="inlineStr"/>
-      <c r="Y16" s="8" t="inlineStr"/>
-    </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="13" t="n">
+      <c r="V22" s="9" t="inlineStr">
+        <is>
+          <t>① FF·CL에서 보증·손실부담 관련 충당 인식요건(현재의무·유출가능성·신뢰성 있는 추정) 검토 ② '성능 개선을 통해 달성 가능하다'는 등 낙관적 예상만으로 충당 미계상하지 않았는지 점검 ③ 손실부담계약(회피불가능원가 vs 기대효익) 여부 판단 ④ 최선의 추정치·현재가치 측정 문서화</t>
+        </is>
+      </c>
+      <c r="W22" s="9" t="inlineStr">
+        <is>
+          <t>보증·손실부담 충당 인식요건이 충족되는가?; 충당부채 측정·결론이 문서화되어 있는가?; 낙관적 예상만을 근거로 충당부채를 미적립하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X22" s="9" t="inlineStr"/>
+      <c r="Y22" s="9" t="inlineStr"/>
+      <c r="Z22" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 14.16, K-IFRS 1037호(손실부담계약: 회피불가능원가&gt;기대효익)</t>
+        </is>
+      </c>
+      <c r="AA22" s="11" t="inlineStr">
+        <is>
+          <t>KSA 540(회계추정 감사 — 기댓값·최선추정치 검토)</t>
+        </is>
+      </c>
+      <c r="AB22" s="11" t="inlineStr">
+        <is>
+          <t>KICPA-2022-16(1심 패소 후 낙관적 판단으로 소송충당·자산인식 지연)</t>
+        </is>
+      </c>
+      <c r="AC22" s="11" t="inlineStr"/>
+      <c r="AD22" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목38(공유)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>충당부채의 인식·측정과 우발부채 공시</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>L4-02</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>소송 관련 충당부채</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>소송충당 미계상</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 K사</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>1심 패소 후 소송충당 미계상·은폐</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 K사</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>전 최대주주가 제기한 대여금 반환 청구소송 1심에서 패소하였음에도 영업 및 투자유치에 악영향을 미칠까 우려하여 외부감사인에게 이를 은폐하고 소송충당부채를 계상하지 않음</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr"/>
-      <c r="J17" s="8" t="inlineStr">
+      <c r="I23" s="9" t="inlineStr"/>
+      <c r="J23" s="9" t="inlineStr">
         <is>
           <t>소송</t>
         </is>
       </c>
-      <c r="K17" s="8" t="inlineStr">
+      <c r="K23" s="9" t="inlineStr">
         <is>
           <t>충당; 패소; 소송충당</t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>소송</t>
         </is>
       </c>
-      <c r="M17" s="8" t="inlineStr">
+      <c r="M23" s="9" t="inlineStr">
         <is>
           <t>충당; 패소; 추정</t>
         </is>
       </c>
-      <c r="N17" s="8" t="inlineStr">
+      <c r="N23" s="9" t="inlineStr">
         <is>
           <t>진행중; 미계상</t>
         </is>
       </c>
-      <c r="O17" s="8" t="inlineStr">
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1037호</t>
         </is>
       </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>소송·분쟁 충당 인식 검토 문서화</t>
-        </is>
-      </c>
-      <c r="Q17" s="8" t="inlineStr">
-        <is>
-          <t>소송 결과 반영·충당 결론 보강</t>
-        </is>
-      </c>
-      <c r="R17" s="8" t="inlineStr"/>
-      <c r="S17" s="8" t="inlineStr">
+      <c r="P23" s="9" t="inlineStr">
+        <is>
+          <t>소송·분쟁 충당 인식 검토를 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>소송 결과 반영·충당 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R23" s="9" t="inlineStr"/>
+      <c r="S23" s="9" t="inlineStr">
         <is>
           <t>충당부채; 우발부채·약정</t>
         </is>
       </c>
-      <c r="T17" s="8" t="inlineStr">
+      <c r="T23" s="9" t="inlineStr">
         <is>
           <t>소송; 충당; 우발</t>
         </is>
       </c>
-      <c r="U17" s="8" t="inlineStr">
+      <c r="U23" s="9" t="inlineStr">
         <is>
           <t>FF; CL</t>
         </is>
       </c>
-      <c r="V17" s="8" t="inlineStr">
-        <is>
-          <t>① 소송·분쟁 현황·진행 단계 확인 ② 패소 가능성·충당 인식 여부 ③ 소송 관련 충당·공시 결론</t>
-        </is>
-      </c>
-      <c r="W17" s="8" t="inlineStr">
-        <is>
-          <t>소송·분쟁에 대한 충당 인식이 검토되었는가?; 패소 가능성 반영 결론이 있는가?</t>
-        </is>
-      </c>
-      <c r="X17" s="8" t="inlineStr"/>
-      <c r="Y17" s="8" t="inlineStr"/>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="13" t="n">
+      <c r="V23" s="9" t="inlineStr">
+        <is>
+          <t>① 소송·분쟁 현황·진행 단계 확인(변호사조회서) ② 패소 가능성·충당 인식 여부, 1심 패소를 은폐하지 않았는지 확인(경영진 서면진술과 대사) ③ 위약금·지연이자 등 부수채무 반영 여부 ④ 소송 관련 충당·공시 결론</t>
+        </is>
+      </c>
+      <c r="W23" s="9" t="inlineStr">
+        <is>
+          <t>소송·분쟁에 대한 충당 인식이 검토되었는가?; 패소 가능성 반영 결론이 있는가?; 1심 패소 사실을 감사인에게 은폐하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X23" s="9" t="inlineStr"/>
+      <c r="Y23" s="9" t="inlineStr"/>
+      <c r="Z23" s="11" t="inlineStr">
+        <is>
+          <t>실무지침 실14.11(1심 판결 내용은 충당부채 측정에 반영), K-IFRS 1010호 문단9(보고기간후사건 — 소송 확정은 수정요 사건)</t>
+        </is>
+      </c>
+      <c r="AA23" s="11" t="inlineStr">
+        <is>
+          <t>KSA 501 문단9-12(법률고문 질문·조회), KSA 560(후속사건)</t>
+        </is>
+      </c>
+      <c r="AB23" s="11" t="inlineStr">
+        <is>
+          <t>FSS2008-24(제1호 펀드 패소 후 제2·3호 펀드도 추정 가능함에도 우발부채로만 처리); KICPA-2024-25(차입약정 관련 소송 패소 결과·위약금·지연이자 미반영)</t>
+        </is>
+      </c>
+      <c r="AC23" s="11" t="inlineStr">
+        <is>
+          <t>질의회신 1481(소송충당부채의 조정여부 — 원본 PDF 빈 문서 확인, 재확보 필요)</t>
+        </is>
+      </c>
+      <c r="AD23" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목38(공유)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>충당부채의 인식·측정과 우발부채 공시</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C24" s="9" t="inlineStr">
         <is>
           <t>L4-03</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>연대·약정 우발부채 공시</t>
         </is>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>우발부채 미공시</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>금감원 회계위반예시 L사</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>구두 합의로 연대의무 소멸 판단·우발부채 미공시</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>금감원 2026년 회계위반 예시 L사</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>광고사업권 컨소시엄 대표사업자로서 부사업자와 연대의무를 부담하였는데, 부사업자와의 구두 협의만으로 연대의무를 더 이상 부담하지 않는다고 판단하여 우발부채를 공시하지 않음(발주자와의 최초 계약은 변경되지 않아 연대의무는 유효)</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr"/>
-      <c r="J18" s="8" t="inlineStr">
+      <c r="I24" s="9" t="inlineStr"/>
+      <c r="J24" s="9" t="inlineStr">
         <is>
           <t>우발</t>
         </is>
       </c>
-      <c r="K18" s="8" t="inlineStr">
+      <c r="K24" s="9" t="inlineStr">
         <is>
           <t>연대; 약정; 지급보증; 공시</t>
         </is>
       </c>
-      <c r="L18" s="8" t="inlineStr">
+      <c r="L24" s="9" t="inlineStr">
         <is>
           <t>우발; 공시</t>
         </is>
       </c>
-      <c r="M18" s="8" t="inlineStr">
+      <c r="M24" s="9" t="inlineStr">
         <is>
           <t>연대; 약정; 지급보증</t>
         </is>
       </c>
-      <c r="N18" s="8" t="inlineStr">
+      <c r="N24" s="9" t="inlineStr">
         <is>
           <t>구두만; 공시 없음</t>
         </is>
       </c>
-      <c r="O18" s="8" t="inlineStr">
+      <c r="O24" s="9" t="inlineStr">
         <is>
           <t>K-IFRS 1037호; 1001호</t>
         </is>
       </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>연대·약정 우발부채 공시 검토</t>
-        </is>
-      </c>
-      <c r="Q18" s="8" t="inlineStr">
-        <is>
-          <t>계약 변경 여부·우발부채 공시 결론 보강</t>
-        </is>
-      </c>
-      <c r="R18" s="8" t="inlineStr"/>
-      <c r="S18" s="8" t="inlineStr">
+      <c r="P24" s="9" t="inlineStr">
+        <is>
+          <t>연대·약정 우발부채 공시 검토를 문서화 바랍니다(구두 합의만으로 계약상 의무 소멸을 인정하지 않았는지 포함)</t>
+        </is>
+      </c>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>계약 변경 여부·우발부채 공시 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R24" s="9" t="inlineStr"/>
+      <c r="S24" s="9" t="inlineStr">
         <is>
           <t>충당부채; 우발부채·약정</t>
         </is>
       </c>
-      <c r="T18" s="8" t="inlineStr">
+      <c r="T24" s="9" t="inlineStr">
         <is>
           <t>우발; 약정; 지급보증</t>
         </is>
       </c>
-      <c r="U18" s="8" t="inlineStr">
+      <c r="U24" s="9" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="V18" s="8" t="inlineStr">
-        <is>
-          <t>① CL에서 연대·지급보증·약정 우발부채 식별 ② 유출가능성·공시 요건 검토 ③ 계약 변경(구두 합의 등) 반영·공시 확인</t>
-        </is>
-      </c>
-      <c r="W18" s="8" t="inlineStr">
-        <is>
-          <t>연대·약정 우발부채가 식별·공시되었는가?; 지급보증·약정 변경이 반영되었는가?</t>
-        </is>
-      </c>
-      <c r="X18" s="8" t="inlineStr"/>
-      <c r="Y18" s="8" t="inlineStr"/>
+      <c r="V24" s="9" t="inlineStr">
+        <is>
+          <t>① CL에서 연대·지급보증·약정 우발부채 식별(투자자간 계약상 위약매수청구권 등 변형된 형태 포함) ② 유출가능성·공시 요건 검토 ③ 구두 협의·묵시적 해지만으로 연대의무 소멸을 인정하지 않았는지 확인 — 서면 계약 변경 여부가 확인되지 않는 한 최초 계약상 의무는 유효 ④ 계약 변경(구두 합의 등) 반영·공시 확인</t>
+        </is>
+      </c>
+      <c r="W24" s="9" t="inlineStr">
+        <is>
+          <t>연대·약정 우발부채가 식별·공시되었는가?; 지급보증·약정 변경이 반영되었는가?; 구두 협의만으로 계약상 연대의무 소멸을 인정하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X24" s="9" t="inlineStr"/>
+      <c r="Y24" s="9" t="inlineStr"/>
+      <c r="Z24" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1001호 문단114, 1037호 문단10·18</t>
+        </is>
+      </c>
+      <c r="AA24" s="11" t="inlineStr">
+        <is>
+          <t>KSA 501 문단6-8, KSA 505(외부조회)</t>
+        </is>
+      </c>
+      <c r="AB24" s="11" t="inlineStr">
+        <is>
+          <t>FSS2606-09(투자자간 계약 위약매수청구권 Penalty Put-Option); FSS2112-17(옵션 이면계약으로 780억원 대출금 인수의무 미기재)</t>
+        </is>
+      </c>
+      <c r="AC24" s="11" t="inlineStr"/>
+      <c r="AD24" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목38(공유)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>충당부채의 인식·측정과 우발부채 공시</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>L4-04</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>담보제공자산(자기 채무 담보) 및 제공받은 담보 주석 공시</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>담보제공자산 주석 미기재·과소기재</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>금감원·한공회 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>자기 채무의 담보로 제공한 자산(부동산·투자주식·매출채권·예금 등) 또는 특수관계자로부터 받은 담보(신탁 우선수익권 등)의 주석누락·과소기재</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>검토누락</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>담보제공자산 유의적인 경우</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>담보</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>질권; 신탁; 우선수익권; 근저당; 담보제공</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>담보 공시</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>담보 내역 공시; 말소 확인</t>
+        </is>
+      </c>
+      <c r="N25" s="9" t="inlineStr">
+        <is>
+          <t>담보 미기재</t>
+        </is>
+      </c>
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 제2장; K-IFRS 1016호; 1107호</t>
+        </is>
+      </c>
+      <c r="P25" s="9" t="inlineStr">
+        <is>
+          <t>자기 채무 담보로 제공한 자산 및 특수관계자로부터 받은 담보의 주석 공시 여부를 등기부등본·금융기관조회서와 대사하여 검토 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>담보제공자산 내역(설정액·말소여부) 공시를 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R25" s="9" t="inlineStr"/>
+      <c r="S25" s="9" t="inlineStr">
+        <is>
+          <t>충당부채; 우발부채·약정</t>
+        </is>
+      </c>
+      <c r="T25" s="9" t="inlineStr">
+        <is>
+          <t>담보; 질권; 신탁; 근저당; 지급보증</t>
+        </is>
+      </c>
+      <c r="U25" s="9" t="inlineStr">
+        <is>
+          <t>CL; A; F; G</t>
+        </is>
+      </c>
+      <c r="V25" s="9" t="inlineStr">
+        <is>
+          <t>① 자기 채무 담보로 제공된 자산(부동산·투자주식·매출채권·정기예금 등) 목록 확인 ② 등기부등본·금융기관조회서·은행연합회 자료와 담보설정 내역 대사 ③ 대출 상환·신탁등기 말소 후에도 담보제공 사실이 잘못 유지 기재되지 않았는지 확인 ④ 특수관계자로부터 받은 담보(신탁 우선수익권 등)도 공시대상인지 확인</t>
+        </is>
+      </c>
+      <c r="W25" s="9" t="inlineStr">
+        <is>
+          <t>담보로 제공된 자산이 주석에 공시되었는가?; 대출 상환·담보 말소 후에도 담보제공 사실이 잘못 유지 기재되지 않았는가?; 특수관계자로부터 받은 담보도 공시대상으로 검토하였는가?</t>
+        </is>
+      </c>
+      <c r="X25" s="9" t="inlineStr">
+        <is>
+          <t>현금및현금성자산; 유형자산; 투자부동산; 매출채권</t>
+        </is>
+      </c>
+      <c r="Y25" s="9" t="inlineStr">
+        <is>
+          <t>제공하거나 제공받은 담보가 없는 경우</t>
+        </is>
+      </c>
+      <c r="Z25" s="11" t="inlineStr">
+        <is>
+          <t>일반기업회계기준 2.85·실무지침 실2.20, 제10장 문단10.48⑶, K-IFRS 1016호 문단74, 1107호 문단14·36</t>
+        </is>
+      </c>
+      <c r="AA25" s="11" t="inlineStr">
+        <is>
+          <t>KSA 505(외부조회 — 은행조회서 완전성), KSA 501</t>
+        </is>
+      </c>
+      <c r="AB25" s="11" t="inlineStr">
+        <is>
+          <t>KICPA-2020-26(자기 담보제공 과소기재); FSS2505-14(종속기업투자주식·부동산 담보); FSS2606-10(제공받은 담보 신탁 우선수익권); FSS2008-30(대출 상환 후에도 담보제공 사실 잘못 유지 기재)</t>
+        </is>
+      </c>
+      <c r="AC25" s="11" t="inlineStr"/>
+      <c r="AD25" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목28: 실재성 및 권리관계(등기부등본) 검토내역 누락 시 지적</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>충당부채의 인식·측정과 우발부채 공시</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>L4-05</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여충당부채 측정</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여충당부채 과소계상</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>금감원 감리지적사례 종합</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>보험수리적 기법 대신 퇴직금 추계액에 근속 1년미만 제외·임의 비율(예: 80%) 적용, 특수관계자(대주주 임원)와의 이면합의로 장기간 미계상 후 소급 일시인식</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>결론미비</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr"/>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>충당부채; 보험수리적; 추계액</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>보험수리적 가정</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>보험수리적 평가; 계리보고서</t>
+        </is>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>추계액 임의비율; 이면합의</t>
+        </is>
+      </c>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>K-IFRS 1019호</t>
+        </is>
+      </c>
+      <c r="P26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여충당부채 측정방법(보험수리적 기법 여부) 및 주요가정 검토를 문서화 바랍니다</t>
+        </is>
+      </c>
+      <c r="Q26" s="9" t="inlineStr">
+        <is>
+          <t>계리보고서 주요가정(할인율 등) 검토·재계산 결론을 보강 바랍니다</t>
+        </is>
+      </c>
+      <c r="R26" s="9" t="inlineStr"/>
+      <c r="S26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여충당부채</t>
+        </is>
+      </c>
+      <c r="T26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여; 충당부채; 계리; 보험수리적</t>
+        </is>
+      </c>
+      <c r="U26" s="9" t="inlineStr">
+        <is>
+          <t>R; FF</t>
+        </is>
+      </c>
+      <c r="V26" s="9" t="inlineStr">
+        <is>
+          <t>① 퇴직급여충당부채가 보험수리적 기법(계리보고서)에 근거하여 측정되었는지, 퇴직금 추계액에 임의 비율을 적용하지 않았는지 확인 ② 근속 1년미만 직원 제외 등 임의적 조정 여부 점검 ③ 특수관계자(대주주·임원)와의 이면합의로 장기간 미계상 후 소급 일시인식 등 이익조정 목적 여부 확인 ④ 계리보고서 주요가정(할인율·임금상승률) 검토절차 수행 여부 확인</t>
+        </is>
+      </c>
+      <c r="W26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여충당부채가 보험수리적 기법으로 측정되었는가?; 퇴직금 추계액에 임의 비율을 적용하지 않았는가?; 특수관계자와의 이면합의로 퇴직급여충당부채 인식이 지연되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="X26" s="9" t="inlineStr">
+        <is>
+          <t>퇴직급여충당부채</t>
+        </is>
+      </c>
+      <c r="Y26" s="9" t="inlineStr">
+        <is>
+          <t>확정기여형 퇴직급여제도만 운영하는 경우</t>
+        </is>
+      </c>
+      <c r="Z26" s="11" t="inlineStr">
+        <is>
+          <t>K-IFRS 1019호 문단66, 개념체계 문단4.27</t>
+        </is>
+      </c>
+      <c r="AA26" s="11" t="inlineStr">
+        <is>
+          <t>KSA 540 문단8-9(전문가 이용), KSA 620(감사인측 전문가 — 계리인 활용시)</t>
+        </is>
+      </c>
+      <c r="AB26" s="11" t="inlineStr">
+        <is>
+          <t>FSS2206-12(보험수리적 기법 대신 퇴직금 추계액+1년미만 제외+80% 임의적용); FSS2409-09(특수관계자(대주주 임원)와의 이면합의로 장기간 미계상 후 소급 일시인식)</t>
+        </is>
+      </c>
+      <c r="AC26" s="11" t="inlineStr"/>
+      <c r="AD26" s="11" t="inlineStr">
+        <is>
+          <t>QC 사후심리 항목36(판관비/인건비 R): 계리평가보고서의 주요가정(할인율 등)에 대한 검토절차 미실시 시 지적</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y18"/>
+  <autoFilter ref="A1:AD26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2686,85 +4179,178 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>리뷰노트 유형</t>
         </is>
       </c>
+      <c r="B1" s="17" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>검토누락</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>조서에 해당 지적유형·검토 절차 흔적이 없음 → [4대중점·검토누락]</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>결론미비</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>검토는 있으나 감사결론·근거가 불충분 → [4대중점·결론미비]</t>
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="17" t="n"/>
+      <c r="B4" s="17" t="n"/>
+    </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>중요성</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>관련 계정·거래가 중요성 미만이면 중요도 '중'으로 하향 또는 지적 생략</t>
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="17" t="n"/>
+      <c r="B6" s="17" t="n"/>
+    </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>구체적 검토지침</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>review_procedure — 항목별 ①②③ 검토절차 (보도자료·감리지적사례 기반)</t>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>review_procedure — 항목별 ①②③④ 검토절차 (보도자료·감리지적사례·QC심리점검표 기반)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>조서 인덱스</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>related_sheet_codes — FY2026 계정과목 조서 인덱스 (C, E, SAJ 등)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>리뷰노트 규칙</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>checklist_id별 1건 · [4대중점·검토누락/결론미비] · 조서 인덱스만 표기</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="n"/>
+      <c r="B10" s="17" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>[신규] standard_paragraphs</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>K-IFRS·일반기업회계기준 구체적 조문·문단 번호 인용</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>[신규] audit_standard_ref</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>관련 회계감사기준(KSA) 조항 — 위험평가·회계추정·특수관계자·그룹감사 등</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>[신규] additional_case_refs</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>금감원·한공회 감리지적사례 추가 사례(2021~2026년, 사례코드+요약)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>[신규] qna_refs</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>한국회계기준원 질의회신 인용(번호+주제)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>[신규] qc_checklist_ref</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>한울 사전/사후심리 체크리스트(QC) 연계 항목·미흡판정기준</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="n"/>
+      <c r="B16" s="17" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>고도화 이력</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>2026-07 — 금감원·한공회 감리지적사례 480건, 질의회신 2,148건, 회계감사기준 전문, 일반기업회계기준 33개장, K-IFRS 실무사례해설, 사전/사후심리 체크리스트를 근거자료로 보강. 기존 checklist_id·golden_set_ids·탐지 키워드는 보존, 신규 세부항목은 각 이슈 말미에 추가.</t>
         </is>
       </c>
     </row>

</xml_diff>